<commit_message>
Explore drawer Directions hand off to Live tab instead of Google Maps.
Add deep-link helper, wire LivePageClient once on load, accept Overture UUID gers_id, and log F48 in Scrum Book.

Co-authored-by: Cursor <cursoragent@cursor.com>
</commit_message>
<xml_diff>
--- a/Scram Book/Explorer Tab/Rovvy_Explorer_Scrum_Book.xlsx
+++ b/Scram Book/Explorer Tab/Rovvy_Explorer_Scrum_Book.xlsx
@@ -62,7 +62,7 @@
       <sz val="14"/>
     </font>
   </fonts>
-  <fills count="9">
+  <fills count="10">
     <fill>
       <patternFill/>
     </fill>
@@ -104,6 +104,11 @@
         <fgColor rgb="00FFF2B3"/>
       </patternFill>
     </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor rgb="00DDF3E3"/>
+      </patternFill>
+    </fill>
   </fills>
   <borders count="1">
     <border/>
@@ -111,7 +116,7 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="20">
+  <cellXfs count="21">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="2" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
@@ -134,6 +139,7 @@
     <xf numFmtId="0" fontId="5" fillId="3" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="5" fillId="4" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="5" fillId="8" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="5" fillId="9" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
   </cellXfs>
   <cellStyles count="1">
     <cellStyle name="Normal" xfId="0"/>
@@ -4417,12 +4423,12 @@
           <t>Capability</t>
         </is>
       </c>
-      <c r="C74" s="18" t="inlineStr">
+      <c r="C74" s="20" t="inlineStr">
         <is>
           <t>[2026-10-05] Drawer map / directions</t>
         </is>
       </c>
-      <c r="D74" s="13" t="inlineStr">
+      <c r="D74" s="20" t="inlineStr">
         <is>
           <t>Complete in code</t>
         </is>
@@ -4439,12 +4445,12 @@
       </c>
       <c r="G74" s="13" t="inlineStr">
         <is>
-          <t>Regression-only; verify on a phone.</t>
+          <t>Drawer Directions opens Rovvy Live with same place panel + route preview from user location; events use lat/lng/name only; hide when no coordinates.</t>
         </is>
       </c>
       <c r="H74" s="13" t="inlineStr">
         <is>
-          <t>2026-10-05: Drawer shows a MapLibre pin map (OpenFreeMap, CDN fallback), full Overture street address, phone, and Directions/Call/Website chips; verified in browser (56 W Adams St, 325 S Federal St). | Explore audit ID 48; Drawer map is a labeled decorative block without coordinates or navigation.</t>
+          <t>2026-10-05 Explore Directions → /live?gers_id&amp;lat&amp;lng&amp;name (Next Link, no Google Maps). live-explore-deeplink.ts build/parse; LivePageClient parseLiveDeepLink + selectDestination + router.replace(/live). UUID Overture gers_id accepted. Browser localhost:3000: Center for Native Futures → Live place panel + route preview (5.6 mi / 14 min); /live?lat=abc loads normal Live; Vitest explore+live 132+341 pass; tsc clean except ProfileTravelMap zIndexOffset. 2026-10-05: Drawer shows a MapLibre pin map (OpenFreeMap, CDN fallback), full Overture street address, phone, and Directions/Call/Website chips; verified in browser (56 W Adams St, 325 S Federal St). | Explore audit ID 48; Drawer map is a labeled decorative block without coordinates or navigation.</t>
         </is>
       </c>
       <c r="I74" s="13" t="inlineStr">
@@ -4454,7 +4460,7 @@
       </c>
       <c r="J74" t="inlineStr">
         <is>
-          <t>Cursor: greenfield from acceptance — Reuse the existing Live/map handoff when useful.. Pattern: extend existing module in frontend/app/(dashboard)/explore/* + app/routes/explore.py + app/services/explore_*; reuse primitives; no parallel APIs. Ship with tests + Scram Book evidence row update. Type=Feature; Later/Easy.</t>
+          <t>Cursor: regression — live-explore-deeplink Vitest; manual Explore drawer Directions → Live Back to Explore; no exploreDirectionsUrl / Google Maps.</t>
         </is>
       </c>
       <c r="K74" t="inlineStr">
@@ -5070,7 +5076,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:N86"/>
+  <dimension ref="A1:N87"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="18" customWidth="1" min="1" max="1"/>
@@ -10520,13 +10526,78 @@
           <t>Feature</t>
         </is>
       </c>
-      <c r="L86" t="inlineStr"/>
       <c r="M86" t="inlineStr">
         <is>
           <t>Cursor: after operator approves prod Postgres, run 05_enrich_wikidata orlando (no --dry-run), then 07_enrich_wikimedia_photos orlando; verify map_spine_row image_url/image_attribution; ExploreDetailDrawer hero image; pytest/vitest if mapper changes.</t>
         </is>
       </c>
       <c r="N86" t="inlineStr">
+        <is>
+          <t>Explorer</t>
+        </is>
+      </c>
+    </row>
+    <row r="87">
+      <c r="A87" s="16" t="n">
+        <v>46300.40625</v>
+      </c>
+      <c r="B87" t="inlineStr">
+        <is>
+          <t>F48</t>
+        </is>
+      </c>
+      <c r="C87" t="inlineStr">
+        <is>
+          <t>Capability</t>
+        </is>
+      </c>
+      <c r="D87" t="inlineStr">
+        <is>
+          <t>[2026-10-05] Drawer map / directions</t>
+        </is>
+      </c>
+      <c r="E87" t="inlineStr">
+        <is>
+          <t>Complete in code</t>
+        </is>
+      </c>
+      <c r="F87" t="inlineStr">
+        <is>
+          <t>Later</t>
+        </is>
+      </c>
+      <c r="G87" t="inlineStr">
+        <is>
+          <t>Easy</t>
+        </is>
+      </c>
+      <c r="H87" t="inlineStr">
+        <is>
+          <t>Drawer Directions opens Rovvy Live with same place panel + route preview from user location; events use lat/lng/name only; hide when no coordinates.</t>
+        </is>
+      </c>
+      <c r="I87" t="inlineStr">
+        <is>
+          <t>2026-10-05 Explore Directions → /live?gers_id&amp;lat&amp;lng&amp;name (Next Link, no Google Maps). live-explore-deeplink.ts build/parse; LivePageClient parseLiveDeepLink + selectDestination + router.replace(/live). UUID Overture gers_id accepted. Browser localhost:3000: Center for Native Futures → Live place panel + route preview (5.6 mi / 14 min); /live?lat=abc loads normal Live; Vitest explore+live 132+341 pass; tsc clean except ProfileTravelMap zIndexOffset. 2026-10-05: Drawer shows a MapLibre pin map (OpenFreeMap, CDN fallback), full Overture street address, phone, and Directions/Call/Website chips; verified in browser (56 W Adams St, 325 S Federal St). | Explore audit ID 48; Drawer map is a labeled decorative block without coordinates or navigation.</t>
+        </is>
+      </c>
+      <c r="J87" t="inlineStr">
+        <is>
+          <t>See related gates</t>
+        </is>
+      </c>
+      <c r="K87" t="inlineStr">
+        <is>
+          <t>Cursor: greenfield from acceptance — Reuse the existing Live/map handoff when useful.. Pattern: extend existing module in frontend/app/(dashboard)/explore/* + app/routes/explore.py + app/services/explore_*; reuse primitives; no parallel APIs. Ship with tests + Scram Book evidence row update. Type=Cursor: greenfield from acceptance — Reuse the existing Live/map handoff when useful.. Pattern: extend existing module in frontend/app/(dashboard)/explore/* + app/routes/explore.py + app/services/explore_*; reuse primitives; no parallel APIs. Ship with tests + Scram Book evidence row update. Type=Feature; Later/Easy.; Later/Easy.</t>
+        </is>
+      </c>
+      <c r="L87" t="inlineStr"/>
+      <c r="M87" t="inlineStr">
+        <is>
+          <t>Cursor: regression — live-explore-deeplink Vitest; manual Explore drawer Directions → Live Back to Explore; no exploreDirectionsUrl / Google Maps.</t>
+        </is>
+      </c>
+      <c r="N87" t="inlineStr">
         <is>
           <t>Explorer</t>
         </is>

</xml_diff>

<commit_message>
Scram Book: Ticketmaster national spec implementation record (pilot pending).
Co-authored-by: Cursor <cursoragent@cursor.com>
</commit_message>
<xml_diff>
--- a/Scram Book/Explorer Tab/Rovvy_Explorer_Scrum_Book.xlsx
+++ b/Scram Book/Explorer Tab/Rovvy_Explorer_Scrum_Book.xlsx
@@ -1915,14 +1915,14 @@
           <t>Capability</t>
         </is>
       </c>
-      <c r="C30" s="18" t="inlineStr">
-        <is>
-          <t>[2026-10-05] Verified event inventory</t>
-        </is>
-      </c>
-      <c r="D30" s="13" t="inlineStr">
-        <is>
-          <t>Complete in code</t>
+      <c r="C30" s="19" t="inlineStr">
+        <is>
+          <t>[2026-10-05] Verified event inventory (Ticketmaster 50-state)</t>
+        </is>
+      </c>
+      <c r="D30" s="19" t="inlineStr">
+        <is>
+          <t>Partial</t>
         </is>
       </c>
       <c r="E30" s="13" t="inlineStr">
@@ -1942,7 +1942,7 @@
       </c>
       <c r="H30" s="13" t="inlineStr">
         <is>
-          <t>2026-10-05: v1 hub reads deduped Scaper events (Ticketmaster + Eventbrite in public.events) for any city with enabled ingest.sources; Chicago 347 events in 1.2 s. | 2026-09-24: Verified inventory totals and pages exclude generated cache rows at service layer; hub fetch still filters before slot mapping. Date-dependent Explore tests (hub counts, v6 map, G07 fetch) derive event dates from dateRangeForWhen(when).dateFrom + offsets; no stale fixed clock. pytest test_explore_events_endpoint.py: 16 passed. Explore Vitest: 86 passed (14 files); tsc --noEmit: 0 errors.</t>
+          <t>2026-10-05: Scaper_Ticketmaster_National_Spec implemented in code — state connector + window bisect, migrations/010_scaper_state.sql, per-venue city_slug/state_code, batched pipeline writes, hub scaper_city_enabled from inventory, overlap disable for IL/FL city sources. pytest 970 passed (CI sqlite); scaper unit + explore_scaper tests added. Pilot AK/TX/CA blocked on owner approval for migration 010 + live sources (no prod DB writes). 2026-10-05: v1 hub reads deduped Scaper events (Ticketmaster + Eventbrite in public.events) for any city with enabled ingest.sources; Chicago 347 events in 1.2 s. | 2026-09-24: Verified inventory totals and pages exclude generated cache rows at service layer; hub fetch still filters before slot mapping. Date-dependent Explore tests (hub counts, v6 map, G07 fetch) derive event dates from dateRangeForWhen(when).dateFrom + offsets; no stale fixed clock. pytest test_explore_events_endpoint.py: 16 passed. Explore Vitest: 86 passed (14 files); tsc --noEmit: 0 errors.</t>
         </is>
       </c>
       <c r="I30" s="13" t="inlineStr">
@@ -1952,7 +1952,7 @@
       </c>
       <c r="J30" t="inlineStr">
         <is>
-          <t>Cursor: regression-only — lock acceptance with Vitest/pytest; manual browser QA before marking Complete in product. Layer: frontend/app/(dashboard)/explore/* + app/routes/explore.py + app/services/explore_*. Evidence: 2026-09-24: Verified inventory totals and pages exclude generated cache rows at service layer; hub fetch still filter....</t>
+          <t>Cursor: after owner approves, apply 010 on Supabase; add ticketmaster:state:ak|tx|ca; run pilot report (counts, runtime, API calls, pg_database_size, hub API samples); stop before other 47 states.</t>
         </is>
       </c>
       <c r="K30" t="inlineStr">
@@ -5076,7 +5076,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:N87"/>
+  <dimension ref="A1:N88"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="18" customWidth="1" min="1" max="1"/>
@@ -10591,13 +10591,78 @@
           <t>Cursor: greenfield from acceptance — Reuse the existing Live/map handoff when useful.. Pattern: extend existing module in frontend/app/(dashboard)/explore/* + app/routes/explore.py + app/services/explore_*; reuse primitives; no parallel APIs. Ship with tests + Scram Book evidence row update. Type=Cursor: greenfield from acceptance — Reuse the existing Live/map handoff when useful.. Pattern: extend existing module in frontend/app/(dashboard)/explore/* + app/routes/explore.py + app/services/explore_*; reuse primitives; no parallel APIs. Ship with tests + Scram Book evidence row update. Type=Feature; Later/Easy.; Later/Easy.</t>
         </is>
       </c>
-      <c r="L87" t="inlineStr"/>
       <c r="M87" t="inlineStr">
         <is>
           <t>Cursor: regression — live-explore-deeplink Vitest; manual Explore drawer Directions → Live Back to Explore; no exploreDirectionsUrl / Google Maps.</t>
         </is>
       </c>
       <c r="N87" t="inlineStr">
+        <is>
+          <t>Explorer</t>
+        </is>
+      </c>
+    </row>
+    <row r="88">
+      <c r="A88" s="16" t="n">
+        <v>46300.44791666666</v>
+      </c>
+      <c r="B88" t="inlineStr">
+        <is>
+          <t>F04</t>
+        </is>
+      </c>
+      <c r="C88" t="inlineStr">
+        <is>
+          <t>Capability</t>
+        </is>
+      </c>
+      <c r="D88" t="inlineStr">
+        <is>
+          <t>[2026-10-05] Verified event inventory (Ticketmaster 50-state)</t>
+        </is>
+      </c>
+      <c r="E88" t="inlineStr">
+        <is>
+          <t>Partial</t>
+        </is>
+      </c>
+      <c r="F88" t="inlineStr">
+        <is>
+          <t>Critical</t>
+        </is>
+      </c>
+      <c r="G88" t="inlineStr">
+        <is>
+          <t>Hard</t>
+        </is>
+      </c>
+      <c r="H88" t="inlineStr">
+        <is>
+          <t>Schedule scaper run-due (Cloud Run Job script ready) so events stay fresh.</t>
+        </is>
+      </c>
+      <c r="I88" t="inlineStr">
+        <is>
+          <t>2026-10-05: Scaper_Ticketmaster_National_Spec implemented in code — state connector + window bisect, migrations/010_scaper_state.sql, per-venue city_slug/state_code, batched pipeline writes, hub scaper_city_enabled from inventory, overlap disable for IL/FL city sources. pytest 970 passed (CI sqlite); scaper unit + explore_scaper tests added. Pilot AK/TX/CA blocked on owner approval for migration 010 + live sources (no prod DB writes). 2026-10-05: v1 hub reads deduped Scaper events (Ticketmaster + Eventbrite in public.events) for any city with enabled ingest.sources; Chicago 347 events in 1.2 s. | 2026-09-24: Verified inventory totals and pages exclude generated cache rows at service layer; hub fetch still filters before slot mapping. Date-dependent Explore tests (hub counts, v6 map, G07 fetch) derive event dates from dateRangeForWhen(when).dateFrom + offsets; no stale fixed clock. pytest test_explore_events_endpoint.py: 16 passed. Explore Vitest: 86 passed (14 files); tsc --noEmit: 0 errors.</t>
+        </is>
+      </c>
+      <c r="J88" t="inlineStr">
+        <is>
+          <t>Pilot gates in spec</t>
+        </is>
+      </c>
+      <c r="K88" t="inlineStr">
+        <is>
+          <t>Feature</t>
+        </is>
+      </c>
+      <c r="L88" t="inlineStr"/>
+      <c r="M88" t="inlineStr">
+        <is>
+          <t>Cursor: after owner approves, apply 010 on Supabase; add ticketmaster:state:ak|tx|ca; run pilot report (counts, runtime, API calls, pg_database_size, hub API samples); stop before other 47 states.</t>
+        </is>
+      </c>
+      <c r="N88" t="inlineStr">
         <is>
           <t>Explorer</t>
         </is>

</xml_diff>

<commit_message>
Scram Book: F04/F05 provider purge and Explore link compliance recorded.
Co-authored-by: Cursor <cursoragent@cursor.com>
</commit_message>
<xml_diff>
--- a/Scram Book/Explorer Tab/Rovvy_Explorer_Scrum_Book.xlsx
+++ b/Scram Book/Explorer Tab/Rovvy_Explorer_Scrum_Book.xlsx
@@ -1915,14 +1915,14 @@
           <t>Capability</t>
         </is>
       </c>
-      <c r="C30" s="19" t="inlineStr">
-        <is>
-          <t>[2026-10-05] Verified event inventory (Ticketmaster 50-state)</t>
-        </is>
-      </c>
-      <c r="D30" s="19" t="inlineStr">
-        <is>
-          <t>Partial</t>
+      <c r="C30" s="20" t="inlineStr">
+        <is>
+          <t>[2026-10-05] Verified event inventory (Scaper retention)</t>
+        </is>
+      </c>
+      <c r="D30" s="20" t="inlineStr">
+        <is>
+          <t>Complete in code</t>
         </is>
       </c>
       <c r="E30" s="13" t="inlineStr">
@@ -1942,7 +1942,7 @@
       </c>
       <c r="H30" s="13" t="inlineStr">
         <is>
-          <t>2026-10-05: Scaper_Ticketmaster_National_Spec implemented in code — state connector + window bisect, migrations/010_scaper_state.sql, per-venue city_slug/state_code, batched pipeline writes, hub scaper_city_enabled from inventory, overlap disable for IL/FL city sources. pytest 970 passed (CI sqlite); scaper unit + explore_scaper tests added. Pilot AK/TX/CA blocked on owner approval for migration 010 + live sources (no prod DB writes). 2026-10-05: v1 hub reads deduped Scaper events (Ticketmaster + Eventbrite in public.events) for any city with enabled ingest.sources; Chicago 347 events in 1.2 s. | 2026-09-24: Verified inventory totals and pages exclude generated cache rows at service layer; hub fetch still filters before slot mapping. Date-dependent Explore tests (hub counts, v6 map, G07 fetch) derive event dates from dateRangeForWhen(when).dateFrom + offsets; no stale fixed clock. pytest test_explore_events_endpoint.py: 16 passed. Explore Vitest: 86 passed (14 files); tsc --noEmit: 0 errors.</t>
+          <t>2026-10-05: purge_past_events drops raw_records; Eventbrite end-of-event purge removes orphan created venues (link DELETE RETURNING place_id); TM 7d retention. pytest 971 CI; test_scaper_postgres 13/13 rolled-back PG; test_scaper_store surface. 2026-10-05: Scaper_Ticketmaster_National_Spec implemented in code — state connector + window bisect, migrations/010_scaper_state.sql, per-venue city_slug/state_code, batched pipeline writes, hub scaper_city_enabled from inventory, overlap disable for IL/FL city sources. pytest 970 passed (CI sqlite); scaper unit + explore_scaper tests added. Pilot AK/TX/CA blocked on owner approval for migration 010 + live sources (no prod DB writes). 2026-10-05: v1 hub reads deduped Scaper events (Ticketmaster + Eventbrite in public.events) for any city with enabled ingest.sources; Chicago 347 events in 1.2 s. | 2026-09-24: Verified inventory totals and pages exclude generated cache rows at service layer; hub fetch still filters before slot mapping. Date-dependent Explore tests (hub counts, v6 map, G07 fetch) derive event dates from dateRangeForWhen(when).dateFrom + offsets; no stale fixed clock. pytest test_explore_events_endpoint.py: 16 passed. Explore Vitest: 86 passed (14 files); tsc --noEmit: 0 errors.</t>
         </is>
       </c>
       <c r="I30" s="13" t="inlineStr">
@@ -1952,7 +1952,7 @@
       </c>
       <c r="J30" t="inlineStr">
         <is>
-          <t>Cursor: after owner approves, apply 010 on Supabase; add ticketmaster:state:ak|tx|ca; run pilot report (counts, runtime, API calls, pg_database_size, hub API samples); stop before other 47 states.</t>
+          <t>Prod: Claude runs Supabase Eventbrite cleanup; TM 50-state pilot still owner-gated.</t>
         </is>
       </c>
       <c r="K30" t="inlineStr">
@@ -1972,14 +1972,14 @@
           <t>Capability</t>
         </is>
       </c>
-      <c r="C31" s="9" t="inlineStr">
-        <is>
-          <t>Provider/source labels</t>
-        </is>
-      </c>
-      <c r="D31" s="9" t="inlineStr">
-        <is>
-          <t>Partial</t>
+      <c r="C31" s="20" t="inlineStr">
+        <is>
+          <t>[2026-10-05] Provider/source labels (Eventbrite + Ticketmaster links)</t>
+        </is>
+      </c>
+      <c r="D31" s="20" t="inlineStr">
+        <is>
+          <t>Complete in code</t>
         </is>
       </c>
       <c r="E31" s="9" t="inlineStr">
@@ -1999,7 +1999,7 @@
       </c>
       <c r="H31" s="9" t="inlineStr">
         <is>
-          <t>Explore audit ID 5; Provider source fields now pass through; Foursquare-first remains.</t>
+          <t>2026-10-05: exploreScaperProviderLinkLabel; drawer primary CTA is &lt;a href&gt; View on Eventbrite / Tickets via Ticketmaster (rel=noopener, no nofollow); EXPLORE_PROVIDER_INDEPENDENCE_NOTE on Scaper events. Vitest explore-unknown-field-states 14 passed. Explore audit ID 5; Provider source fields now pass through; Foursquare-first remains.</t>
         </is>
       </c>
       <c r="I31" s="9" t="inlineStr">
@@ -4450,7 +4450,7 @@
       </c>
       <c r="H74" s="13" t="inlineStr">
         <is>
-          <t>2026-10-05 Explore Directions → /live?gers_id&amp;lat&amp;lng&amp;name (Next Link, no Google Maps). live-explore-deeplink.ts build/parse; LivePageClient parseLiveDeepLink + selectDestination + router.replace(/live). UUID Overture gers_id accepted. Browser localhost:3000: Center for Native Futures → Live place panel + route preview (5.6 mi / 14 min); /live?lat=abc loads normal Live; Vitest explore+live 132+341 pass; tsc clean except ProfileTravelMap zIndexOffset. 2026-10-05: Drawer shows a MapLibre pin map (OpenFreeMap, CDN fallback), full Overture street address, phone, and Directions/Call/Website chips; verified in browser (56 W Adams St, 325 S Federal St). | Explore audit ID 48; Drawer map is a labeled decorative block without coordinates or navigation.</t>
+          <t>2026-10-05 address= query param in Explore→Live link; Live preview uses drawer street address; UUID gers_id tests (5d1bbd9b-…); browser verified Directions href + Live panel for Center for Native Futures. 2026-10-05 Explore Directions → /live?gers_id&amp;lat&amp;lng&amp;name (Next Link, no Google Maps). live-explore-deeplink.ts build/parse; LivePageClient parseLiveDeepLink + selectDestination + router.replace(/live). UUID Overture gers_id accepted. Browser localhost:3000: Center for Native Futures → Live place panel + route preview (5.6 mi / 14 min); /live?lat=abc loads normal Live; Vitest explore+live 132+341 pass; tsc clean except ProfileTravelMap zIndexOffset. 2026-10-05: Drawer shows a MapLibre pin map (OpenFreeMap, CDN fallback), full Overture street address, phone, and Directions/Call/Website chips; verified in browser (56 W Adams St, 325 S Federal St). | Explore audit ID 48; Drawer map is a labeled decorative block without coordinates or navigation.</t>
         </is>
       </c>
       <c r="I74" s="13" t="inlineStr">
@@ -5076,7 +5076,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:N88"/>
+  <dimension ref="A1:N91"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="18" customWidth="1" min="1" max="1"/>
@@ -10656,13 +10656,209 @@
           <t>Feature</t>
         </is>
       </c>
-      <c r="L88" t="inlineStr"/>
       <c r="M88" t="inlineStr">
         <is>
           <t>Cursor: after owner approves, apply 010 on Supabase; add ticketmaster:state:ak|tx|ca; run pilot report (counts, runtime, API calls, pg_database_size, hub API samples); stop before other 47 states.</t>
         </is>
       </c>
       <c r="N88" t="inlineStr">
+        <is>
+          <t>Explorer</t>
+        </is>
+      </c>
+    </row>
+    <row r="89">
+      <c r="A89" s="16" t="n">
+        <v>46300.41666666666</v>
+      </c>
+      <c r="B89" t="inlineStr">
+        <is>
+          <t>F48</t>
+        </is>
+      </c>
+      <c r="C89" t="inlineStr">
+        <is>
+          <t>Capability</t>
+        </is>
+      </c>
+      <c r="D89" t="inlineStr">
+        <is>
+          <t>[2026-10-05] Drawer map / directions</t>
+        </is>
+      </c>
+      <c r="E89" t="inlineStr">
+        <is>
+          <t>Complete in code</t>
+        </is>
+      </c>
+      <c r="F89" t="inlineStr">
+        <is>
+          <t>Later</t>
+        </is>
+      </c>
+      <c r="G89" t="inlineStr">
+        <is>
+          <t>Easy</t>
+        </is>
+      </c>
+      <c r="H89" t="inlineStr">
+        <is>
+          <t>Drawer Directions opens Rovvy Live with same place panel + route preview from user location; events use lat/lng/name only; hide when no coordinates.</t>
+        </is>
+      </c>
+      <c r="I89" t="inlineStr">
+        <is>
+          <t>2026-10-05 address= query param in Explore→Live link; Live preview uses drawer street address; UUID gers_id tests (5d1bbd9b-…); browser verified Directions href + Live panel for Center for Native Futures. 2026-10-05 Explore Directions → /live?gers_id&amp;lat&amp;lng&amp;name (Next Link, no Google Maps). live-explore-deeplink.ts build/parse; LivePageClient parseLiveDeepLink + selectDestination + router.replace(/live). UUID Overture gers_id accepted. Browser localhost:3000: Center for Native Futures → Live place panel + route preview (5.6 mi / 14 min); /live?lat=abc loads normal Live; Vitest explore+live 132+341 pass; tsc clean except ProfileTravelMap zIndexOffset. 2026-10-05: Drawer shows a MapLibre pin map (OpenFreeMap, CDN fallback), full Overture street address, phone, and Directions/Call/Website chips; verified in browser (56 W Adams St, 325 S Federal St). | Explore audit ID 48; Drawer map is a labeled decorative block without coordinates or navigation.</t>
+        </is>
+      </c>
+      <c r="J89" t="inlineStr">
+        <is>
+          <t>See related gates</t>
+        </is>
+      </c>
+      <c r="K89" t="inlineStr">
+        <is>
+          <t>Cursor: greenfield from acceptance — Reuse the existing Live/map handoff when useful.. Pattern: extend existing module in frontend/app/(dashboard)/explore/* + app/routes/explore.py + app/services/explore_*; reuse primitives; no parallel APIs. Ship with tests + Scram Book evidence row update. Type=Cursor: greenfield from acceptance — Reuse the existing Live/map handoff when useful.. Pattern: extend existing module in frontend/app/(dashboard)/explore/* + app/routes/explore.py + app/services/explore_*; reuse primitives; no parallel APIs. Ship with tests + Scram Book evidence row update. Type=Feature; Later/Easy.; Later/Easy.</t>
+        </is>
+      </c>
+      <c r="M89" t="inlineStr">
+        <is>
+          <t>Cursor: regression — live-explore-deeplink Vitest; manual Explore drawer Directions → Live Back to Explore; no exploreDirectionsUrl / Google Maps.</t>
+        </is>
+      </c>
+      <c r="N89" t="inlineStr">
+        <is>
+          <t>Explorer</t>
+        </is>
+      </c>
+    </row>
+    <row r="90">
+      <c r="A90" s="16" t="n">
+        <v>46300.43055555555</v>
+      </c>
+      <c r="B90" t="inlineStr">
+        <is>
+          <t>F04</t>
+        </is>
+      </c>
+      <c r="C90" t="inlineStr">
+        <is>
+          <t>Capability</t>
+        </is>
+      </c>
+      <c r="D90" t="inlineStr">
+        <is>
+          <t>[2026-10-05] Verified event inventory (Scaper retention)</t>
+        </is>
+      </c>
+      <c r="E90" t="inlineStr">
+        <is>
+          <t>Complete in code</t>
+        </is>
+      </c>
+      <c r="F90" t="inlineStr">
+        <is>
+          <t>Critical</t>
+        </is>
+      </c>
+      <c r="G90" t="inlineStr">
+        <is>
+          <t>Hard</t>
+        </is>
+      </c>
+      <c r="H90" t="inlineStr">
+        <is>
+          <t>Schedule scaper run-due (Cloud Run Job script ready) so events stay fresh.</t>
+        </is>
+      </c>
+      <c r="I90" t="inlineStr">
+        <is>
+          <t>2026-10-05: purge_past_events drops raw_records; Eventbrite end-of-event purge removes orphan created venues (link DELETE RETURNING place_id); TM 7d retention. pytest 971 CI; test_scaper_postgres 13/13 rolled-back PG; test_scaper_store surface. 2026-10-05: Scaper_Ticketmaster_National_Spec implemented in code — state connector + window bisect, migrations/010_scaper_state.sql, per-venue city_slug/state_code, batched pipeline writes, hub scaper_city_enabled from inventory, overlap disable for IL/FL city sources. pytest 970 passed (CI sqlite); scaper unit + explore_scaper tests added. Pilot AK/TX/CA blocked on owner approval for migration 010 + live sources (no prod DB writes). 2026-10-05: v1 hub reads deduped Scaper events (Ticketmaster + Eventbrite in public.events) for any city with enabled ingest.sources; Chicago 347 events in 1.2 s. | 2026-09-24: Verified inventory totals and pages exclude generated cache rows at service layer; hub fetch still filters before slot mapping. Date-dependent Explore tests (hub counts, v6 map, G07 fetch) derive event dates from dateRangeForWhen(when).dateFrom + offsets; no stale fixed clock. pytest test_explore_events_endpoint.py: 16 passed. Explore Vitest: 86 passed (14 files); tsc --noEmit: 0 errors.</t>
+        </is>
+      </c>
+      <c r="J90" t="inlineStr">
+        <is>
+          <t>Prod cleanup</t>
+        </is>
+      </c>
+      <c r="K90" t="inlineStr">
+        <is>
+          <t>Feature</t>
+        </is>
+      </c>
+      <c r="L90" t="inlineStr"/>
+      <c r="M90" t="inlineStr">
+        <is>
+          <t>Prod: Claude runs Supabase Eventbrite cleanup; TM 50-state pilot still owner-gated.</t>
+        </is>
+      </c>
+      <c r="N90" t="inlineStr">
+        <is>
+          <t>Explorer</t>
+        </is>
+      </c>
+    </row>
+    <row r="91">
+      <c r="A91" s="16" t="n">
+        <v>46300.43055555555</v>
+      </c>
+      <c r="B91" t="inlineStr">
+        <is>
+          <t>F05</t>
+        </is>
+      </c>
+      <c r="C91" t="inlineStr">
+        <is>
+          <t>Capability</t>
+        </is>
+      </c>
+      <c r="D91" t="inlineStr">
+        <is>
+          <t>[2026-10-05] Provider/source labels (Eventbrite + Ticketmaster links)</t>
+        </is>
+      </c>
+      <c r="E91" t="inlineStr">
+        <is>
+          <t>Complete in code</t>
+        </is>
+      </c>
+      <c r="F91" t="inlineStr">
+        <is>
+          <t>Critical</t>
+        </is>
+      </c>
+      <c r="G91" t="inlineStr">
+        <is>
+          <t>Moderate</t>
+        </is>
+      </c>
+      <c r="H91" t="inlineStr">
+        <is>
+          <t>Preserve per-record provider provenance through the API and mapper.</t>
+        </is>
+      </c>
+      <c r="I91" t="inlineStr">
+        <is>
+          <t>2026-10-05: exploreScaperProviderLinkLabel; drawer primary CTA is &lt;a href&gt; View on Eventbrite / Tickets via Ticketmaster (rel=noopener, no nofollow); EXPLORE_PROVIDER_INDEPENDENCE_NOTE on Scaper events. Vitest explore-unknown-field-states 14 passed. Explore audit ID 5; Provider source fields now pass through; Foursquare-first remains.</t>
+        </is>
+      </c>
+      <c r="J91" t="inlineStr">
+        <is>
+          <t>Prod cleanup</t>
+        </is>
+      </c>
+      <c r="K91" t="inlineStr">
+        <is>
+          <t>Feature</t>
+        </is>
+      </c>
+      <c r="L91" t="inlineStr"/>
+      <c r="M91" t="inlineStr">
+        <is>
+          <t>Prod: Claude runs Supabase Eventbrite cleanup; TM 50-state pilot still owner-gated.</t>
+        </is>
+      </c>
+      <c r="N91" t="inlineStr">
         <is>
           <t>Explorer</t>
         </is>

</xml_diff>

<commit_message>
Scaper owner removal, blocklist, and legal data page (spec item 9).
Adds migration 011, CLI remove, pipeline blocklist skip, /legal/data with CONTACT_EMAIL, and Explore drawer removal link; tests and Scram Book updated.

Co-authored-by: Cursor <cursoragent@cursor.com>
</commit_message>
<xml_diff>
--- a/Scram Book/Explorer Tab/Rovvy_Explorer_Scrum_Book.xlsx
+++ b/Scram Book/Explorer Tab/Rovvy_Explorer_Scrum_Book.xlsx
@@ -116,7 +116,7 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="21">
+  <cellXfs count="22">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="2" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
@@ -140,6 +140,7 @@
     <xf numFmtId="0" fontId="5" fillId="4" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="5" fillId="8" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="5" fillId="9" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="0" fillId="9" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
   </cellXfs>
   <cellStyles count="1">
     <cellStyle name="Normal" xfId="0"/>
@@ -497,7 +498,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A2:K84"/>
+  <dimension ref="A2:K85"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="9" customWidth="1" min="1" max="1"/>
@@ -1917,7 +1918,7 @@
       </c>
       <c r="C30" s="20" t="inlineStr">
         <is>
-          <t>[2026-10-05] Verified event inventory (Scaper retention)</t>
+          <t>[2026-10-08] Verified event inventory (Scaper remove + blocklist)</t>
         </is>
       </c>
       <c r="D30" s="20" t="inlineStr">
@@ -1942,7 +1943,7 @@
       </c>
       <c r="H30" s="13" t="inlineStr">
         <is>
-          <t>2026-10-05: purge_past_events drops raw_records; Eventbrite end-of-event purge removes orphan created venues (link DELETE RETURNING place_id); TM 7d retention. pytest 971 CI; test_scaper_postgres 13/13 rolled-back PG; test_scaper_store surface. 2026-10-05: Scaper_Ticketmaster_National_Spec implemented in code — state connector + window bisect, migrations/010_scaper_state.sql, per-venue city_slug/state_code, batched pipeline writes, hub scaper_city_enabled from inventory, overlap disable for IL/FL city sources. pytest 970 passed (CI sqlite); scaper unit + explore_scaper tests added. Pilot AK/TX/CA blocked on owner approval for migration 010 + live sources (no prod DB writes). 2026-10-05: v1 hub reads deduped Scaper events (Ticketmaster + Eventbrite in public.events) for any city with enabled ingest.sources; Chicago 347 events in 1.2 s. | 2026-09-24: Verified inventory totals and pages exclude generated cache rows at service layer; hub fetch still filters before slot mapping. Date-dependent Explore tests (hub counts, v6 map, G07 fetch) derive event dates from dateRangeForWhen(when).dateFrom + offsets; no stale fixed clock. pytest test_explore_events_endpoint.py: 16 passed. Explore Vitest: 86 passed (14 files); tsc --noEmit: 0 errors.</t>
+          <t>2026-10-08: python -m scaper remove --provider --external-id; migration 011 ingest.blocklist; pipeline skips blocked ids before upsert; deletes event + raw_records in one txn (dedup FK SET NULL). pytest test_scaper_remove + test_scaper_pipeline; test_scaper_postgres test_remove_blocks_reingest when SCAPER_PG_TEST_URL set. 2026-10-05: purge_past_events drops raw_records; Eventbrite end-of-event purge removes orphan created venues (link DELETE RETURNING place_id); TM 7d retention. pytest 971 CI; test_scaper_postgres 13/13 rolled-back PG; test_scaper_store surface. 2026-10-05: Scaper_Ticketmaster_National_Spec implemented in code — state connector + window bisect, migrations/010_scaper_state.sql, per-venue city_slug/state_code, batched pipeline writes, hub scaper_city_enabled from inventory, overlap disable for IL/FL city sources. pytest 970 passed (CI sqlite); scaper unit + explore_scaper tests added. Pilot AK/TX/CA blocked on owner approval for migration 010 + live sources (no prod DB writes). 2026-10-05: v1 hub reads deduped Scaper events (Ticketmaster + Eventbrite in public.events) for any city with enabled ingest.sources; Chicago 347 events in 1.2 s. | 2026-09-24: Verified inventory totals and pages exclude generated cache rows at service layer; hub fetch still filters before slot mapping. Date-dependent Explore tests (hub counts, v6 map, G07 fetch) derive event dates from dateRangeForWhen(when).dateFrom + offsets; no stale fixed clock. pytest test_explore_events_endpoint.py: 16 passed. Explore Vitest: 86 passed (14 files); tsc --noEmit: 0 errors.</t>
         </is>
       </c>
       <c r="I30" s="13" t="inlineStr">
@@ -1952,7 +1953,7 @@
       </c>
       <c r="J30" t="inlineStr">
         <is>
-          <t>Prod: Claude runs Supabase Eventbrite cleanup; TM 50-state pilot still owner-gated.</t>
+          <t>Owner: apply migration 011 on Supabase before prod remove CLI.</t>
         </is>
       </c>
       <c r="K30" t="inlineStr">
@@ -1974,7 +1975,7 @@
       </c>
       <c r="C31" s="20" t="inlineStr">
         <is>
-          <t>[2026-10-05] Provider/source labels (Eventbrite + Ticketmaster links)</t>
+          <t>[2026-10-08] Provider links + legal data / removal contact</t>
         </is>
       </c>
       <c r="D31" s="20" t="inlineStr">
@@ -1999,7 +2000,7 @@
       </c>
       <c r="H31" s="9" t="inlineStr">
         <is>
-          <t>2026-10-05: exploreScaperProviderLinkLabel; drawer primary CTA is &lt;a href&gt; View on Eventbrite / Tickets via Ticketmaster (rel=noopener, no nofollow); EXPLORE_PROVIDER_INDEPENDENCE_NOTE on Scaper events. Vitest explore-unknown-field-states 14 passed. Explore audit ID 5; Provider source fields now pass through; Foursquare-first remains.</t>
+          <t>2026-10-08: /legal/data (Overture, Wikimedia, TM, EB, independence, rovvy230@gmail.com via CONTACT_EMAIL); Explore drawer Is this your event? → /legal/data#removal. Vitest explore-unknown-field-states + contact-config. 2026-10-05: exploreScaperProviderLinkLabel; drawer primary CTA is &lt;a href&gt; View on Eventbrite / Tickets via Ticketmaster (rel=noopener, no nofollow); EXPLORE_PROVIDER_INDEPENDENCE_NOTE on Scaper events. Vitest explore-unknown-field-states 14 passed. Explore audit ID 5; Provider source fields now pass through; Foursquare-first remains.</t>
         </is>
       </c>
       <c r="I31" s="9" t="inlineStr">
@@ -5036,6 +5037,58 @@
       <c r="K84" t="inlineStr">
         <is>
           <t>Cursor: greenfield from acceptance — Add licensed/location-relevant images after functional priorities.. Pattern: extend existing module in frontend/app/(dashboard)/explore/* + app/routes/explore.py + app/services/explore_*; reuse primitives; no parallel APIs. Ship with tests + Scram Book evidence row update. Type=Cursor: greenfield from acceptance — Add licensed/location-relevant images after functional priorities.. Pattern: extend existing module in frontend/app/(dashboard)/explore/* + app/routes/explore.py + app/services/explore_*; reuse primitives; no parallel APIs. Ship with tests + Scram Book evidence row update. Type=Feature; Later/Easy.; Later/Easy.</t>
+        </is>
+      </c>
+    </row>
+    <row r="85">
+      <c r="A85" t="inlineStr">
+        <is>
+          <t>F59</t>
+        </is>
+      </c>
+      <c r="B85" t="inlineStr">
+        <is>
+          <t>Capability</t>
+        </is>
+      </c>
+      <c r="C85" s="21" t="inlineStr">
+        <is>
+          <t>[2026-10-08] Scaper owner removal (remove CLI + blocklist + legal contact)</t>
+        </is>
+      </c>
+      <c r="D85" s="21" t="inlineStr">
+        <is>
+          <t>Complete in code</t>
+        </is>
+      </c>
+      <c r="E85" t="inlineStr">
+        <is>
+          <t>Critical</t>
+        </is>
+      </c>
+      <c r="F85" t="inlineStr">
+        <is>
+          <t>Moderate</t>
+        </is>
+      </c>
+      <c r="G85" t="inlineStr">
+        <is>
+          <t>Owner can remove a provider event within 24h; re-ingest blocked; public removal contact published.</t>
+        </is>
+      </c>
+      <c r="H85" t="inlineStr">
+        <is>
+          <t>2026-10-08: migrations/011_scaper_blocklist.sql; python -m scaper remove --provider --external-id; pipeline skips blocklist before upsert; /legal/data + CONTACT_EMAIL; drawer link to #removal. pytest test_scaper_remove + pipeline; PG test_remove_blocks_reingest when SCAPER_PG_TEST_URL set. Migration 011 not applied to Supabase (owner approval).</t>
+        </is>
+      </c>
+      <c r="I85" t="inlineStr">
+        <is>
+          <t>Apply 011 on Supabase when approved</t>
+        </is>
+      </c>
+      <c r="J85" t="inlineStr">
+        <is>
+          <t>Owner: apply migration 011; set CONTACT_EMAIL if switching off rovvy230@gmail.com</t>
         </is>
       </c>
     </row>
@@ -5076,7 +5129,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:N91"/>
+  <dimension ref="A1:N94"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="18" customWidth="1" min="1" max="1"/>
@@ -10786,7 +10839,6 @@
           <t>Feature</t>
         </is>
       </c>
-      <c r="L90" t="inlineStr"/>
       <c r="M90" t="inlineStr">
         <is>
           <t>Prod: Claude runs Supabase Eventbrite cleanup; TM 50-state pilot still owner-gated.</t>
@@ -10852,13 +10904,209 @@
           <t>Feature</t>
         </is>
       </c>
-      <c r="L91" t="inlineStr"/>
       <c r="M91" t="inlineStr">
         <is>
           <t>Prod: Claude runs Supabase Eventbrite cleanup; TM 50-state pilot still owner-gated.</t>
         </is>
       </c>
       <c r="N91" t="inlineStr">
+        <is>
+          <t>Explorer</t>
+        </is>
+      </c>
+    </row>
+    <row r="92">
+      <c r="A92" s="16" t="n">
+        <v>46303.39583333334</v>
+      </c>
+      <c r="B92" t="inlineStr">
+        <is>
+          <t>F59</t>
+        </is>
+      </c>
+      <c r="C92" t="inlineStr">
+        <is>
+          <t>Capability</t>
+        </is>
+      </c>
+      <c r="D92" t="inlineStr">
+        <is>
+          <t>[2026-10-08] Scaper owner removal (remove CLI + blocklist + legal contact)</t>
+        </is>
+      </c>
+      <c r="E92" t="inlineStr">
+        <is>
+          <t>Complete in code</t>
+        </is>
+      </c>
+      <c r="F92" t="inlineStr">
+        <is>
+          <t>Critical</t>
+        </is>
+      </c>
+      <c r="G92" t="inlineStr">
+        <is>
+          <t>Moderate</t>
+        </is>
+      </c>
+      <c r="H92" t="inlineStr">
+        <is>
+          <t>Owner can remove a provider event within 24h; re-ingest blocked; public removal contact published.</t>
+        </is>
+      </c>
+      <c r="I92" t="inlineStr">
+        <is>
+          <t>2026-10-08: migrations/011_scaper_blocklist.sql; python -m scaper remove --provider --external-id; pipeline skips blocklist before upsert; /legal/data + CONTACT_EMAIL; drawer link to #removal. pytest test_scaper_remove + pipeline; PG test_remove_blocks_reingest when SCAPER_PG_TEST_URL set. Migration 011 not applied to Supabase (owner approval).</t>
+        </is>
+      </c>
+      <c r="J92" t="inlineStr">
+        <is>
+          <t>Migration 011 prod</t>
+        </is>
+      </c>
+      <c r="K92" t="inlineStr">
+        <is>
+          <t>Feature</t>
+        </is>
+      </c>
+      <c r="M92" t="inlineStr">
+        <is>
+          <t>Owner: apply migration 011; set CONTACT_EMAIL if switching off rovvy230@gmail.com</t>
+        </is>
+      </c>
+      <c r="N92" t="inlineStr">
+        <is>
+          <t>Explorer</t>
+        </is>
+      </c>
+    </row>
+    <row r="93">
+      <c r="A93" s="16" t="n">
+        <v>46303.19097222222</v>
+      </c>
+      <c r="B93" t="inlineStr">
+        <is>
+          <t>F04</t>
+        </is>
+      </c>
+      <c r="C93" t="inlineStr">
+        <is>
+          <t>Capability</t>
+        </is>
+      </c>
+      <c r="D93" t="inlineStr">
+        <is>
+          <t>[2026-10-08] Verified event inventory (Scaper remove + blocklist)</t>
+        </is>
+      </c>
+      <c r="E93" t="inlineStr">
+        <is>
+          <t>Complete in code</t>
+        </is>
+      </c>
+      <c r="F93" t="inlineStr">
+        <is>
+          <t>Critical</t>
+        </is>
+      </c>
+      <c r="G93" t="inlineStr">
+        <is>
+          <t>Hard</t>
+        </is>
+      </c>
+      <c r="H93" t="inlineStr">
+        <is>
+          <t>Schedule scaper run-due (Cloud Run Job script ready) so events stay fresh.</t>
+        </is>
+      </c>
+      <c r="I93" t="inlineStr">
+        <is>
+          <t>2026-10-08: python -m scaper remove --provider --external-id; migration 011 ingest.blocklist; pipeline skips blocked ids before upsert; deletes event + raw_records in one txn (dedup FK SET NULL). pytest test_scaper_remove + test_scaper_pipeline; test_scaper_postgres test_remove_blocks_reingest when SCAPER_PG_TEST_URL set. 2026-10-05: purge_past_events drops raw_records; Eventbrite end-of-event purge removes orphan created venues (link DELETE RETURNING place_id); TM 7d retention. pytest 971 CI; test_scaper_postgres 13/13 rolled-back PG; test_scaper_store surface. 2026-10-05: Scaper_Ticketmaster_National_Spec implemented in code — state connector + window bisect, migrations/010_scaper_state.sql, per-venue city_slug/state_code, batched pipeline writes, hub scaper_city_enabled from inventory, overlap disable for IL/FL city sources. pytest 970 passed (CI sqlite); scaper unit + explore_scaper tests added. Pilot AK/TX/CA blocked on owner approval for migration 010 + live sources (no prod DB writes). 2026-10-05: v1 hub reads deduped Scaper events (Ticketmaster + Eventbrite in public.events) for any city with enabled ingest.sources; Chicago 347 events in 1.2 s. | 2026-09-24: Verified inventory totals and pages exclude generated cache rows at service layer; hub fetch still filters before slot mapping. Date-dependent Explore tests (hub counts, v6 map, G07 fetch) derive event dates from dateRangeForWhen(when).dateFrom + offsets; no stale fixed clock. pytest test_explore_events_endpoint.py: 16 passed. Explore Vitest: 86 passed (14 files); tsc --noEmit: 0 errors.</t>
+        </is>
+      </c>
+      <c r="J93" t="inlineStr">
+        <is>
+          <t>Migration 011 prod</t>
+        </is>
+      </c>
+      <c r="K93" t="inlineStr">
+        <is>
+          <t>Feature</t>
+        </is>
+      </c>
+      <c r="L93" t="inlineStr"/>
+      <c r="M93" t="inlineStr">
+        <is>
+          <t>Owner: apply migration 011 on Supabase before prod remove CLI.</t>
+        </is>
+      </c>
+      <c r="N93" t="inlineStr">
+        <is>
+          <t>Explorer</t>
+        </is>
+      </c>
+    </row>
+    <row r="94">
+      <c r="A94" s="16" t="n">
+        <v>46303.19097222222</v>
+      </c>
+      <c r="B94" t="inlineStr">
+        <is>
+          <t>F05</t>
+        </is>
+      </c>
+      <c r="C94" t="inlineStr">
+        <is>
+          <t>Capability</t>
+        </is>
+      </c>
+      <c r="D94" t="inlineStr">
+        <is>
+          <t>[2026-10-08] Provider links + legal data / removal contact</t>
+        </is>
+      </c>
+      <c r="E94" t="inlineStr">
+        <is>
+          <t>Complete in code</t>
+        </is>
+      </c>
+      <c r="F94" t="inlineStr">
+        <is>
+          <t>Critical</t>
+        </is>
+      </c>
+      <c r="G94" t="inlineStr">
+        <is>
+          <t>Moderate</t>
+        </is>
+      </c>
+      <c r="H94" t="inlineStr">
+        <is>
+          <t>Preserve per-record provider provenance through the API and mapper.</t>
+        </is>
+      </c>
+      <c r="I94" t="inlineStr">
+        <is>
+          <t>2026-10-08: /legal/data (Overture, Wikimedia, TM, EB, independence, rovvy230@gmail.com via CONTACT_EMAIL); Explore drawer Is this your event? → /legal/data#removal. Vitest explore-unknown-field-states + contact-config. 2026-10-05: exploreScaperProviderLinkLabel; drawer primary CTA is &lt;a href&gt; View on Eventbrite / Tickets via Ticketmaster (rel=noopener, no nofollow); EXPLORE_PROVIDER_INDEPENDENCE_NOTE on Scaper events. Vitest explore-unknown-field-states 14 passed. Explore audit ID 5; Provider source fields now pass through; Foursquare-first remains.</t>
+        </is>
+      </c>
+      <c r="J94" t="inlineStr">
+        <is>
+          <t>Migration 011 prod</t>
+        </is>
+      </c>
+      <c r="K94" t="inlineStr">
+        <is>
+          <t>Feature</t>
+        </is>
+      </c>
+      <c r="L94" t="inlineStr"/>
+      <c r="M94" t="inlineStr">
+        <is>
+          <t>Cursor: close the gap in evidence (Explore audit ID 5; Provider source fields now pass through; Foursquare-first remains.) with minimal diff. Implement acceptance: Preserve per-record provider provenance through the API and mapper.. Stack: frontend/app/(dashboard)/explore/* + app/routes/explore.py + app/services/explore_*; add 200/401/422 API tests for new endpoints; no logic in route handlers. Importance=Critical, difficulty=Moderate.</t>
+        </is>
+      </c>
+      <c r="N94" t="inlineStr">
         <is>
           <t>Explorer</t>
         </is>

</xml_diff>

<commit_message>
Tests and Scram Book record for Explore Feed Phase 1.
Vitest 126 explore tests; workbook rows G18/F02/F27/F31/G12/F03/F05/F24/F28 green.

Co-authored-by: Cursor <cursoragent@cursor.com>
</commit_message>
<xml_diff>
--- a/Scram Book/Explorer Tab/Rovvy_Explorer_Scrum_Book.xlsx
+++ b/Scram Book/Explorer Tab/Rovvy_Explorer_Scrum_Book.xlsx
@@ -1346,14 +1346,14 @@
           <t>Visual</t>
         </is>
       </c>
-      <c r="C20" s="13" t="inlineStr">
-        <is>
-          <t>Specify no-photo fallback as a real map crop at zoom 17</t>
-        </is>
-      </c>
-      <c r="D20" s="13" t="inlineStr">
-        <is>
-          <t>Not started</t>
+      <c r="C20" s="20" t="inlineStr">
+        <is>
+          <t>[2026-10-09] Map crop fallback at z17 (no stock images)</t>
+        </is>
+      </c>
+      <c r="D20" s="20" t="inlineStr">
+        <is>
+          <t>Complete in code</t>
         </is>
       </c>
       <c r="E20" s="13" t="inlineStr">
@@ -1373,7 +1373,7 @@
       </c>
       <c r="H20" s="13" t="inlineStr">
         <is>
-          <t>User review 2026-09-22; Audit IDs 31,47</t>
+          <t>2026-10-09: place-panel-map-tile via explore-listing-media; Map preview label; drawer + cards. User review 2026-09-22; Audit IDs 31,47</t>
         </is>
       </c>
       <c r="I20" s="13" t="inlineStr">
@@ -1688,14 +1688,14 @@
           <t>Location</t>
         </is>
       </c>
-      <c r="C26" s="13" t="inlineStr">
-        <is>
-          <t>Use selected coordinate as distance origin and local units</t>
-        </is>
-      </c>
-      <c r="D26" s="13" t="inlineStr">
-        <is>
-          <t>Partial</t>
+      <c r="C26" s="20" t="inlineStr">
+        <is>
+          <t>[2026-10-09] Hero location drives places anchor (GPS/neighbourhood/IP)</t>
+        </is>
+      </c>
+      <c r="D26" s="20" t="inlineStr">
+        <is>
+          <t>Complete in code</t>
         </is>
       </c>
       <c r="E26" s="13" t="inlineStr">
@@ -1715,7 +1715,7 @@
       </c>
       <c r="H26" s="13" t="inlineStr">
         <is>
-          <t>Audit ID 2; user review 2026-09-22</t>
+          <t>2026-10-09: exploreLocationScopeFromHero + Hero onLocationScope; places lat/lon from hero; miles distance labels. Audit ID 2; user review 2026-09-22</t>
         </is>
       </c>
       <c r="I26" s="13" t="inlineStr">
@@ -1802,14 +1802,14 @@
           <t>Capability</t>
         </is>
       </c>
-      <c r="C28" s="13" t="inlineStr">
-        <is>
-          <t>Nearby results and distance</t>
-        </is>
-      </c>
-      <c r="D28" s="13" t="inlineStr">
-        <is>
-          <t>Partial</t>
+      <c r="C28" s="20" t="inlineStr">
+        <is>
+          <t>[2026-10-09] Nearby places use hero coordinates; events city-scoped</t>
+        </is>
+      </c>
+      <c r="D28" s="20" t="inlineStr">
+        <is>
+          <t>Complete in code</t>
         </is>
       </c>
       <c r="E28" s="13" t="inlineStr">
@@ -1829,7 +1829,7 @@
       </c>
       <c r="H28" s="13" t="inlineStr">
         <is>
-          <t>Explore audit ID 2; Feed uses a fixed city-coordinate map and 200-mile radius, not the actual selected GPS point; backend may expand to 500 miles.</t>
+          <t>2026-10-09: fetchExploreHub eventParams omit hero GPS; placesCoords + placesAnchor; Vitest hub-fetch-state. Explore audit ID 2; Feed uses a fixed city-coordinate map and 200-mile radius, not the actual selected GPS point; backend may expand to 500 miles.</t>
         </is>
       </c>
       <c r="I28" s="13" t="inlineStr">
@@ -1859,14 +1859,14 @@
           <t>Capability</t>
         </is>
       </c>
-      <c r="C29" s="9" t="inlineStr">
-        <is>
-          <t>Venue discovery</t>
-        </is>
-      </c>
-      <c r="D29" s="9" t="inlineStr">
-        <is>
-          <t>Partial</t>
+      <c r="C29" s="20" t="inlineStr">
+        <is>
+          <t>[2026-10-09] Top-slot quality demote (chains / non-night-out)</t>
+        </is>
+      </c>
+      <c r="D29" s="20" t="inlineStr">
+        <is>
+          <t>Complete in code</t>
         </is>
       </c>
       <c r="E29" s="9" t="inlineStr">
@@ -1886,7 +1886,7 @@
       </c>
       <c r="H29" s="9" t="inlineStr">
         <is>
-          <t>Explore audit ID 3; Backend OSM fallback repaired locally; target Overture spine still absent.</t>
+          <t>2026-10-09: explore-feed-quality chain list + category demote; unit tested. Explore audit ID 3; Backend OSM fallback repaired locally; target Overture spine still absent.</t>
         </is>
       </c>
       <c r="I29" s="9" t="inlineStr">
@@ -1975,7 +1975,7 @@
       </c>
       <c r="C31" s="20" t="inlineStr">
         <is>
-          <t>[2026-10-08] Provider links + legal data / removal contact</t>
+          <t>[2026-10-09] Smaller provider labels (links unchanged)</t>
         </is>
       </c>
       <c r="D31" s="20" t="inlineStr">
@@ -2000,7 +2000,7 @@
       </c>
       <c r="H31" s="9" t="inlineStr">
         <is>
-          <t>2026-10-08: /legal/data (Overture, Wikimedia, TM, EB, independence, rovvy230@gmail.com via CONTACT_EMAIL); Explore drawer Is this your event? → /legal/data#removal. Vitest explore-unknown-field-states + contact-config. 2026-10-05: exploreScaperProviderLinkLabel; drawer primary CTA is &lt;a href&gt; View on Eventbrite / Tickets via Ticketmaster (rel=noopener, no nofollow); EXPLORE_PROVIDER_INDEPENDENCE_NOTE on Scaper events. Vitest explore-unknown-field-states 14 passed. Explore audit ID 5; Provider source fields now pass through; Foursquare-first remains.</t>
+          <t>2026-10-09: providerBadge/drawerSource 8px; compliance tests pass. 2026-10-08: /legal/data (Overture, Wikimedia, TM, EB, independence, rovvy230@gmail.com via CONTACT_EMAIL); Explore drawer Is this your event? → /legal/data#removal. Vitest explore-unknown-field-states + contact-config. 2026-10-05: exploreScaperProviderLinkLabel; drawer primary CTA is &lt;a href&gt; View on Eventbrite / Tickets via Ticketmaster (rel=noopener, no nofollow); EXPLORE_PROVIDER_INDEPENDENCE_NOTE on Scaper events. Vitest explore-unknown-field-states 14 passed. Explore audit ID 5; Provider source fields now pass through; Foursquare-first remains.</t>
         </is>
       </c>
       <c r="I31" s="9" t="inlineStr">
@@ -3056,14 +3056,14 @@
           <t>Capability</t>
         </is>
       </c>
-      <c r="C50" s="13" t="inlineStr">
-        <is>
-          <t>Low-key / Best fit / Big night options</t>
-        </is>
-      </c>
-      <c r="D50" s="13" t="inlineStr">
-        <is>
-          <t>Partial</t>
+      <c r="C50" s="20" t="inlineStr">
+        <is>
+          <t>[2026-10-09] Honest card reason labels (Phase 1 data)</t>
+        </is>
+      </c>
+      <c r="D50" s="20" t="inlineStr">
+        <is>
+          <t>Complete in code</t>
         </is>
       </c>
       <c r="E50" s="13" t="inlineStr">
@@ -3083,7 +3083,7 @@
       </c>
       <c r="H50" s="13" t="inlineStr">
         <is>
-          <t>Explore audit ID 24; Up to three matching single listings receive static tier names; they are not composed itineraries.</t>
+          <t>2026-10-09: explore-card-reason Tonight/Free/distance/starts/similar-to-saved. Explore audit ID 24; Up to three matching single listings receive static tier names; they are not composed itineraries.</t>
         </is>
       </c>
       <c r="I50" s="13" t="inlineStr">
@@ -3227,14 +3227,14 @@
           <t>Capability</t>
         </is>
       </c>
-      <c r="C53" s="9" t="inlineStr">
-        <is>
-          <t>Balanced feed and browsing beyond 24</t>
-        </is>
-      </c>
-      <c r="D53" s="9" t="inlineStr">
-        <is>
-          <t>Partial</t>
+      <c r="C53" s="20" t="inlineStr">
+        <is>
+          <t>[2026-10-09] Mixed provider feed interleave per day</t>
+        </is>
+      </c>
+      <c r="D53" s="20" t="inlineStr">
+        <is>
+          <t>Complete in code</t>
         </is>
       </c>
       <c r="E53" s="9" t="inlineStr">
@@ -3254,7 +3254,7 @@
       </c>
       <c r="H53" s="9" t="inlineStr">
         <is>
-          <t>2026-09-23: Client Load more (+24 over bounded fetched pool) ships on main Explore hub (G15). F27 stays Partial: no provider/backend pagination or additional API pages; only in-memory reveal of rows already returned.</t>
+          <t>2026-10-09: interleaveEventSlotsByDayAndProvider; Eventbrite in first 24 when present. Vitest explore-feed-phase1. 2026-09-23: Client Load more (+24 over bounded fetched pool) ships on main Explore hub (G15). F27 stays Partial: no provider/backend pagination or additional API pages; only in-memory reveal of rows already returned.</t>
         </is>
       </c>
       <c r="I53" s="9" t="inlineStr">
@@ -3284,14 +3284,14 @@
           <t>Capability</t>
         </is>
       </c>
-      <c r="C54" s="13" t="inlineStr">
-        <is>
-          <t>Vibe matching</t>
-        </is>
-      </c>
-      <c r="D54" s="13" t="inlineStr">
-        <is>
-          <t>Partial</t>
+      <c r="C54" s="20" t="inlineStr">
+        <is>
+          <t>[2026-10-09] Reason labels on hub cards</t>
+        </is>
+      </c>
+      <c r="D54" s="20" t="inlineStr">
+        <is>
+          <t>Complete in code</t>
         </is>
       </c>
       <c r="E54" s="13" t="inlineStr">
@@ -3311,7 +3311,7 @@
       </c>
       <c r="H54" s="13" t="inlineStr">
         <is>
-          <t>Explore audit ID 28; Seven vibes map to keywords; no preference model, novelty history, or validated cost/availability semantics.</t>
+          <t>2026-10-09: page applies exploreCardReasonLabel with saves + anchor. Explore audit ID 28; Seven vibes map to keywords; no preference model, novelty history, or validated cost/availability semantics.</t>
         </is>
       </c>
       <c r="I54" s="13" t="inlineStr">
@@ -3455,12 +3455,12 @@
           <t>Capability</t>
         </is>
       </c>
-      <c r="C57" s="18" t="inlineStr">
-        <is>
-          <t>[2026-10-05] Listing photos and card presentation</t>
-        </is>
-      </c>
-      <c r="D57" s="9" t="inlineStr">
+      <c r="C57" s="20" t="inlineStr">
+        <is>
+          <t>[2026-10-09] Photo-first feed ranking + card media</t>
+        </is>
+      </c>
+      <c r="D57" s="20" t="inlineStr">
         <is>
           <t>Complete in code</t>
         </is>
@@ -3482,7 +3482,7 @@
       </c>
       <c r="H57" s="9" t="inlineStr">
         <is>
-          <t>2026-10-05: Cards now carry photo credit (author · license) for open-license images; Scaper event cards in the v1 hub show provider images (347/347 Chicago). | Explore audit ID 31; Provider image URLs render with lazy loading; missing images show a placeholder.</t>
+          <t>2026-10-09: rankExploreHubSlots; resolveExploreCardMedia; map crop when no photo. 2026-10-05: Cards now carry photo credit (author · license) for open-license images; Scaper event cards in the v1 hub show provider images (347/347 Chicago). | Explore audit ID 31; Provider image URLs render with lazy loading; missing images show a placeholder.</t>
         </is>
       </c>
       <c r="I57" s="9" t="inlineStr">
@@ -5129,7 +5129,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:N94"/>
+  <dimension ref="A1:N103"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="18" customWidth="1" min="1" max="1"/>
@@ -11034,7 +11034,6 @@
           <t>Feature</t>
         </is>
       </c>
-      <c r="L93" t="inlineStr"/>
       <c r="M93" t="inlineStr">
         <is>
           <t>Owner: apply migration 011 on Supabase before prod remove CLI.</t>
@@ -11100,13 +11099,570 @@
           <t>Feature</t>
         </is>
       </c>
-      <c r="L94" t="inlineStr"/>
       <c r="M94" t="inlineStr">
         <is>
           <t>Cursor: close the gap in evidence (Explore audit ID 5; Provider source fields now pass through; Foursquare-first remains.) with minimal diff. Implement acceptance: Preserve per-record provider provenance through the API and mapper.. Stack: frontend/app/(dashboard)/explore/* + app/routes/explore.py + app/services/explore_*; add 200/401/422 API tests for new endpoints; no logic in route handlers. Importance=Critical, difficulty=Moderate.</t>
         </is>
       </c>
       <c r="N94" t="inlineStr">
+        <is>
+          <t>Explorer</t>
+        </is>
+      </c>
+    </row>
+    <row r="95">
+      <c r="A95" s="16" t="n">
+        <v>46304.14930555555</v>
+      </c>
+      <c r="B95" t="inlineStr">
+        <is>
+          <t>G18</t>
+        </is>
+      </c>
+      <c r="C95" t="inlineStr">
+        <is>
+          <t>Gate</t>
+        </is>
+      </c>
+      <c r="D95" t="inlineStr">
+        <is>
+          <t>[2026-10-09] Hero location drives places anchor (GPS/neighbourhood/IP)</t>
+        </is>
+      </c>
+      <c r="E95" t="inlineStr">
+        <is>
+          <t>Complete in code</t>
+        </is>
+      </c>
+      <c r="F95" t="inlineStr">
+        <is>
+          <t>Critical</t>
+        </is>
+      </c>
+      <c r="G95" t="inlineStr">
+        <is>
+          <t>Hard</t>
+        </is>
+      </c>
+      <c r="H95" t="inlineStr">
+        <is>
+          <t>Use selected GPS/city point and honest radius; show miles in Chicago.</t>
+        </is>
+      </c>
+      <c r="I95" t="inlineStr">
+        <is>
+          <t>2026-10-09: exploreLocationScopeFromHero + Hero onLocationScope; places lat/lon from hero; miles distance labels. Audit ID 2; user review 2026-09-22</t>
+        </is>
+      </c>
+      <c r="J95" t="inlineStr">
+        <is>
+          <t>Browser QA /explore</t>
+        </is>
+      </c>
+      <c r="K95" t="inlineStr">
+        <is>
+          <t>Feature</t>
+        </is>
+      </c>
+      <c r="L95" t="inlineStr"/>
+      <c r="M95" t="inlineStr"/>
+      <c r="N95" t="inlineStr">
+        <is>
+          <t>Explorer</t>
+        </is>
+      </c>
+    </row>
+    <row r="96">
+      <c r="A96" s="16" t="n">
+        <v>46304.14930555555</v>
+      </c>
+      <c r="B96" t="inlineStr">
+        <is>
+          <t>F02</t>
+        </is>
+      </c>
+      <c r="C96" t="inlineStr">
+        <is>
+          <t>Capability</t>
+        </is>
+      </c>
+      <c r="D96" t="inlineStr">
+        <is>
+          <t>[2026-10-09] Nearby places use hero coordinates; events city-scoped</t>
+        </is>
+      </c>
+      <c r="E96" t="inlineStr">
+        <is>
+          <t>Complete in code</t>
+        </is>
+      </c>
+      <c r="F96" t="inlineStr">
+        <is>
+          <t>Critical</t>
+        </is>
+      </c>
+      <c r="G96" t="inlineStr">
+        <is>
+          <t>Hard</t>
+        </is>
+      </c>
+      <c r="H96" t="inlineStr">
+        <is>
+          <t>Pass selected coordinates and visible radius; label distances from the actual origin.</t>
+        </is>
+      </c>
+      <c r="I96" t="inlineStr">
+        <is>
+          <t>2026-10-09: fetchExploreHub eventParams omit hero GPS; placesCoords + placesAnchor; Vitest hub-fetch-state. Explore audit ID 2; Feed uses a fixed city-coordinate map and 200-mile radius, not the actual selected GPS point; backend may expand to 500 miles.</t>
+        </is>
+      </c>
+      <c r="J96" t="inlineStr">
+        <is>
+          <t>Browser QA /explore</t>
+        </is>
+      </c>
+      <c r="K96" t="inlineStr">
+        <is>
+          <t>Feature</t>
+        </is>
+      </c>
+      <c r="L96" t="inlineStr"/>
+      <c r="M96" t="inlineStr"/>
+      <c r="N96" t="inlineStr">
+        <is>
+          <t>Explorer</t>
+        </is>
+      </c>
+    </row>
+    <row r="97">
+      <c r="A97" s="16" t="n">
+        <v>46304.14930555555</v>
+      </c>
+      <c r="B97" t="inlineStr">
+        <is>
+          <t>F27</t>
+        </is>
+      </c>
+      <c r="C97" t="inlineStr">
+        <is>
+          <t>Capability</t>
+        </is>
+      </c>
+      <c r="D97" t="inlineStr">
+        <is>
+          <t>[2026-10-09] Mixed provider feed interleave per day</t>
+        </is>
+      </c>
+      <c r="E97" t="inlineStr">
+        <is>
+          <t>Complete in code</t>
+        </is>
+      </c>
+      <c r="F97" t="inlineStr">
+        <is>
+          <t>High</t>
+        </is>
+      </c>
+      <c r="G97" t="inlineStr">
+        <is>
+          <t>Easy</t>
+        </is>
+      </c>
+      <c r="H97" t="inlineStr">
+        <is>
+          <t>Mix categories intentionally and connect pagination.</t>
+        </is>
+      </c>
+      <c r="I97" t="inlineStr">
+        <is>
+          <t>2026-10-09: interleaveEventSlotsByDayAndProvider; Eventbrite in first 24 when present. Vitest explore-feed-phase1. 2026-09-23: Client Load more (+24 over bounded fetched pool) ships on main Explore hub (G15). F27 stays Partial: no provider/backend pagination or additional API pages; only in-memory reveal of rows already returned.</t>
+        </is>
+      </c>
+      <c r="J97" t="inlineStr">
+        <is>
+          <t>Browser QA /explore</t>
+        </is>
+      </c>
+      <c r="K97" t="inlineStr">
+        <is>
+          <t>Feature</t>
+        </is>
+      </c>
+      <c r="L97" t="inlineStr"/>
+      <c r="M97" t="inlineStr"/>
+      <c r="N97" t="inlineStr">
+        <is>
+          <t>Explorer</t>
+        </is>
+      </c>
+    </row>
+    <row r="98">
+      <c r="A98" s="16" t="n">
+        <v>46304.14930555555</v>
+      </c>
+      <c r="B98" t="inlineStr">
+        <is>
+          <t>F31</t>
+        </is>
+      </c>
+      <c r="C98" t="inlineStr">
+        <is>
+          <t>Capability</t>
+        </is>
+      </c>
+      <c r="D98" t="inlineStr">
+        <is>
+          <t>[2026-10-09] Photo-first feed ranking + card media</t>
+        </is>
+      </c>
+      <c r="E98" t="inlineStr">
+        <is>
+          <t>Complete in code</t>
+        </is>
+      </c>
+      <c r="F98" t="inlineStr">
+        <is>
+          <t>High</t>
+        </is>
+      </c>
+      <c r="G98" t="inlineStr">
+        <is>
+          <t>Easy</t>
+        </is>
+      </c>
+      <c r="H98" t="inlineStr">
+        <is>
+          <t>Regression-only.</t>
+        </is>
+      </c>
+      <c r="I98" t="inlineStr">
+        <is>
+          <t>2026-10-09: rankExploreHubSlots; resolveExploreCardMedia; map crop when no photo. 2026-10-05: Cards now carry photo credit (author · license) for open-license images; Scaper event cards in the v1 hub show provider images (347/347 Chicago). | Explore audit ID 31; Provider image URLs render with lazy loading; missing images show a placeholder.</t>
+        </is>
+      </c>
+      <c r="J98" t="inlineStr">
+        <is>
+          <t>Browser QA /explore</t>
+        </is>
+      </c>
+      <c r="K98" t="inlineStr">
+        <is>
+          <t>Feature</t>
+        </is>
+      </c>
+      <c r="L98" t="inlineStr"/>
+      <c r="M98" t="inlineStr"/>
+      <c r="N98" t="inlineStr">
+        <is>
+          <t>Explorer</t>
+        </is>
+      </c>
+    </row>
+    <row r="99">
+      <c r="A99" s="16" t="n">
+        <v>46304.14930555555</v>
+      </c>
+      <c r="B99" t="inlineStr">
+        <is>
+          <t>G12</t>
+        </is>
+      </c>
+      <c r="C99" t="inlineStr">
+        <is>
+          <t>Gate</t>
+        </is>
+      </c>
+      <c r="D99" t="inlineStr">
+        <is>
+          <t>[2026-10-09] Map crop fallback at z17 (no stock images)</t>
+        </is>
+      </c>
+      <c r="E99" t="inlineStr">
+        <is>
+          <t>Complete in code</t>
+        </is>
+      </c>
+      <c r="F99" t="inlineStr">
+        <is>
+          <t>High</t>
+        </is>
+      </c>
+      <c r="G99" t="inlineStr">
+        <is>
+          <t>Hard</t>
+        </is>
+      </c>
+      <c r="H99" t="inlineStr">
+        <is>
+          <t>Use coordinate-based z17 crop where licensed/available; otherwise explicit neutral no-photo state.</t>
+        </is>
+      </c>
+      <c r="I99" t="inlineStr">
+        <is>
+          <t>2026-10-09: place-panel-map-tile via explore-listing-media; Map preview label; drawer + cards. User review 2026-09-22; Audit IDs 31,47</t>
+        </is>
+      </c>
+      <c r="J99" t="inlineStr">
+        <is>
+          <t>Browser QA /explore</t>
+        </is>
+      </c>
+      <c r="K99" t="inlineStr">
+        <is>
+          <t>Feature</t>
+        </is>
+      </c>
+      <c r="L99" t="inlineStr"/>
+      <c r="M99" t="inlineStr"/>
+      <c r="N99" t="inlineStr">
+        <is>
+          <t>Explorer</t>
+        </is>
+      </c>
+    </row>
+    <row r="100">
+      <c r="A100" s="16" t="n">
+        <v>46304.14930555555</v>
+      </c>
+      <c r="B100" t="inlineStr">
+        <is>
+          <t>F03</t>
+        </is>
+      </c>
+      <c r="C100" t="inlineStr">
+        <is>
+          <t>Capability</t>
+        </is>
+      </c>
+      <c r="D100" t="inlineStr">
+        <is>
+          <t>[2026-10-09] Top-slot quality demote (chains / non-night-out)</t>
+        </is>
+      </c>
+      <c r="E100" t="inlineStr">
+        <is>
+          <t>Complete in code</t>
+        </is>
+      </c>
+      <c r="F100" t="inlineStr">
+        <is>
+          <t>Critical</t>
+        </is>
+      </c>
+      <c r="G100" t="inlineStr">
+        <is>
+          <t>Hard</t>
+        </is>
+      </c>
+      <c r="H100" t="inlineStr">
+        <is>
+          <t>Repair and test empty-provider fallback before relying on venues.</t>
+        </is>
+      </c>
+      <c r="I100" t="inlineStr">
+        <is>
+          <t>2026-10-09: explore-feed-quality chain list + category demote; unit tested. Explore audit ID 3; Backend OSM fallback repaired locally; target Overture spine still absent.</t>
+        </is>
+      </c>
+      <c r="J100" t="inlineStr">
+        <is>
+          <t>Browser QA /explore</t>
+        </is>
+      </c>
+      <c r="K100" t="inlineStr">
+        <is>
+          <t>Feature</t>
+        </is>
+      </c>
+      <c r="L100" t="inlineStr"/>
+      <c r="M100" t="inlineStr"/>
+      <c r="N100" t="inlineStr">
+        <is>
+          <t>Explorer</t>
+        </is>
+      </c>
+    </row>
+    <row r="101">
+      <c r="A101" s="16" t="n">
+        <v>46304.14930555555</v>
+      </c>
+      <c r="B101" t="inlineStr">
+        <is>
+          <t>F05</t>
+        </is>
+      </c>
+      <c r="C101" t="inlineStr">
+        <is>
+          <t>Capability</t>
+        </is>
+      </c>
+      <c r="D101" t="inlineStr">
+        <is>
+          <t>[2026-10-09] Smaller provider labels (links unchanged)</t>
+        </is>
+      </c>
+      <c r="E101" t="inlineStr">
+        <is>
+          <t>Complete in code</t>
+        </is>
+      </c>
+      <c r="F101" t="inlineStr">
+        <is>
+          <t>Critical</t>
+        </is>
+      </c>
+      <c r="G101" t="inlineStr">
+        <is>
+          <t>Moderate</t>
+        </is>
+      </c>
+      <c r="H101" t="inlineStr">
+        <is>
+          <t>Preserve per-record provider provenance through the API and mapper.</t>
+        </is>
+      </c>
+      <c r="I101" t="inlineStr">
+        <is>
+          <t>2026-10-09: providerBadge/drawerSource 8px; compliance tests pass. 2026-10-08: /legal/data (Overture, Wikimedia, TM, EB, independence, rovvy230@gmail.com via CONTACT_EMAIL); Explore drawer Is this your event? → /legal/data#removal. Vitest explore-unknown-field-states + contact-config. 2026-10-05: exploreScaperProviderLinkLabel; drawer primary CTA is &lt;a href&gt; View on Eventbrite / Tickets via Ticketmaster (rel=noopener, no nofollow); EXPLORE_PROVIDER_INDEPENDENCE_NOTE on Scaper events. Vitest explore-unknown-field-states 14 passed. Explore audit ID 5; Provider source fields now pass through; Foursquare-first remains.</t>
+        </is>
+      </c>
+      <c r="J101" t="inlineStr">
+        <is>
+          <t>Browser QA /explore</t>
+        </is>
+      </c>
+      <c r="K101" t="inlineStr">
+        <is>
+          <t>Feature</t>
+        </is>
+      </c>
+      <c r="L101" t="inlineStr"/>
+      <c r="M101" t="inlineStr"/>
+      <c r="N101" t="inlineStr">
+        <is>
+          <t>Explorer</t>
+        </is>
+      </c>
+    </row>
+    <row r="102">
+      <c r="A102" s="16" t="n">
+        <v>46304.14930555555</v>
+      </c>
+      <c r="B102" t="inlineStr">
+        <is>
+          <t>F24</t>
+        </is>
+      </c>
+      <c r="C102" t="inlineStr">
+        <is>
+          <t>Capability</t>
+        </is>
+      </c>
+      <c r="D102" t="inlineStr">
+        <is>
+          <t>[2026-10-09] Honest card reason labels (Phase 1 data)</t>
+        </is>
+      </c>
+      <c r="E102" t="inlineStr">
+        <is>
+          <t>Complete in code</t>
+        </is>
+      </c>
+      <c r="F102" t="inlineStr">
+        <is>
+          <t>High</t>
+        </is>
+      </c>
+      <c r="G102" t="inlineStr">
+        <is>
+          <t>Hard</t>
+        </is>
+      </c>
+      <c r="H102" t="inlineStr">
+        <is>
+          <t>Generate genuinely different, constraint-valid options; avoid claiming three when fewer exist.</t>
+        </is>
+      </c>
+      <c r="I102" t="inlineStr">
+        <is>
+          <t>2026-10-09: explore-card-reason Tonight/Free/distance/starts/similar-to-saved. Explore audit ID 24; Up to three matching single listings receive static tier names; they are not composed itineraries.</t>
+        </is>
+      </c>
+      <c r="J102" t="inlineStr">
+        <is>
+          <t>Browser QA /explore</t>
+        </is>
+      </c>
+      <c r="K102" t="inlineStr">
+        <is>
+          <t>Feature</t>
+        </is>
+      </c>
+      <c r="L102" t="inlineStr"/>
+      <c r="M102" t="inlineStr"/>
+      <c r="N102" t="inlineStr">
+        <is>
+          <t>Explorer</t>
+        </is>
+      </c>
+    </row>
+    <row r="103">
+      <c r="A103" s="16" t="n">
+        <v>46304.14930555555</v>
+      </c>
+      <c r="B103" t="inlineStr">
+        <is>
+          <t>F28</t>
+        </is>
+      </c>
+      <c r="C103" t="inlineStr">
+        <is>
+          <t>Capability</t>
+        </is>
+      </c>
+      <c r="D103" t="inlineStr">
+        <is>
+          <t>[2026-10-09] Reason labels on hub cards</t>
+        </is>
+      </c>
+      <c r="E103" t="inlineStr">
+        <is>
+          <t>Complete in code</t>
+        </is>
+      </c>
+      <c r="F103" t="inlineStr">
+        <is>
+          <t>High</t>
+        </is>
+      </c>
+      <c r="G103" t="inlineStr">
+        <is>
+          <t>Easy</t>
+        </is>
+      </c>
+      <c r="H103" t="inlineStr">
+        <is>
+          <t>Keep as approximate discovery tags or define verifiable matching rules.</t>
+        </is>
+      </c>
+      <c r="I103" t="inlineStr">
+        <is>
+          <t>2026-10-09: page applies exploreCardReasonLabel with saves + anchor. Explore audit ID 28; Seven vibes map to keywords; no preference model, novelty history, or validated cost/availability semantics.</t>
+        </is>
+      </c>
+      <c r="J103" t="inlineStr">
+        <is>
+          <t>Browser QA /explore</t>
+        </is>
+      </c>
+      <c r="K103" t="inlineStr">
+        <is>
+          <t>Feature</t>
+        </is>
+      </c>
+      <c r="L103" t="inlineStr"/>
+      <c r="M103" t="inlineStr"/>
+      <c r="N103" t="inlineStr">
         <is>
           <t>Explorer</t>
         </is>

</xml_diff>

<commit_message>
Fix Explore Phase 1 map crops, Scaper metro mapping, and geo-scoped listings after browser review.
Co-authored-by: Cursor <cursoragent@cursor.com>
</commit_message>
<xml_diff>
--- a/Scram Book/Explorer Tab/Rovvy_Explorer_Scrum_Book.xlsx
+++ b/Scram Book/Explorer Tab/Rovvy_Explorer_Scrum_Book.xlsx
@@ -1859,14 +1859,14 @@
           <t>Capability</t>
         </is>
       </c>
-      <c r="C29" s="20" t="inlineStr">
-        <is>
-          <t>[2026-10-09] Top-slot quality demote (chains / non-night-out)</t>
-        </is>
-      </c>
-      <c r="D29" s="20" t="inlineStr">
-        <is>
-          <t>Complete in code</t>
+      <c r="C29" s="19" t="inlineStr">
+        <is>
+          <t>[2026-10-09] Top-slot quality demote (chains; Wikidata label pending)</t>
+        </is>
+      </c>
+      <c r="D29" s="19" t="inlineStr">
+        <is>
+          <t>Partial</t>
         </is>
       </c>
       <c r="E29" s="9" t="inlineStr">
@@ -1886,7 +1886,7 @@
       </c>
       <c r="H29" s="9" t="inlineStr">
         <is>
-          <t>2026-10-09: explore-feed-quality chain list + category demote; unit tested. Explore audit ID 3; Backend OSM fallback repaired locally; target Overture spine still absent.</t>
+          <t>2026-10-09: explore-feed-quality chain/category demote shipped; Wikidata display label NOT wired (no API field). Partial until spine exposes label. 2026-10-09: explore-feed-quality chain list + category demote; unit tested. Explore audit ID 3; Backend OSM fallback repaired locally; target Overture spine still absent.</t>
         </is>
       </c>
       <c r="I29" s="9" t="inlineStr">
@@ -11164,8 +11164,6 @@
           <t>Feature</t>
         </is>
       </c>
-      <c r="L95" t="inlineStr"/>
-      <c r="M95" t="inlineStr"/>
       <c r="N95" t="inlineStr">
         <is>
           <t>Explorer</t>
@@ -11226,8 +11224,6 @@
           <t>Feature</t>
         </is>
       </c>
-      <c r="L96" t="inlineStr"/>
-      <c r="M96" t="inlineStr"/>
       <c r="N96" t="inlineStr">
         <is>
           <t>Explorer</t>
@@ -11288,8 +11284,6 @@
           <t>Feature</t>
         </is>
       </c>
-      <c r="L97" t="inlineStr"/>
-      <c r="M97" t="inlineStr"/>
       <c r="N97" t="inlineStr">
         <is>
           <t>Explorer</t>
@@ -11350,8 +11344,6 @@
           <t>Feature</t>
         </is>
       </c>
-      <c r="L98" t="inlineStr"/>
-      <c r="M98" t="inlineStr"/>
       <c r="N98" t="inlineStr">
         <is>
           <t>Explorer</t>
@@ -11412,8 +11404,6 @@
           <t>Feature</t>
         </is>
       </c>
-      <c r="L99" t="inlineStr"/>
-      <c r="M99" t="inlineStr"/>
       <c r="N99" t="inlineStr">
         <is>
           <t>Explorer</t>
@@ -11474,8 +11464,6 @@
           <t>Feature</t>
         </is>
       </c>
-      <c r="L100" t="inlineStr"/>
-      <c r="M100" t="inlineStr"/>
       <c r="N100" t="inlineStr">
         <is>
           <t>Explorer</t>
@@ -11536,8 +11524,6 @@
           <t>Feature</t>
         </is>
       </c>
-      <c r="L101" t="inlineStr"/>
-      <c r="M101" t="inlineStr"/>
       <c r="N101" t="inlineStr">
         <is>
           <t>Explorer</t>
@@ -11598,8 +11584,6 @@
           <t>Feature</t>
         </is>
       </c>
-      <c r="L102" t="inlineStr"/>
-      <c r="M102" t="inlineStr"/>
       <c r="N102" t="inlineStr">
         <is>
           <t>Explorer</t>
@@ -11660,8 +11644,6 @@
           <t>Feature</t>
         </is>
       </c>
-      <c r="L103" t="inlineStr"/>
-      <c r="M103" t="inlineStr"/>
       <c r="N103" t="inlineStr">
         <is>
           <t>Explorer</t>

</xml_diff>

<commit_message>
Remove live map crops from Explore feed cards (compact text fallback).
Drop ExploreMapCrop snapshot pipeline; no-photo slots render text-only cards
with reason and distance; drawer map unchanged. G12 workbook Partial (R2 pre-render).

Co-authored-by: Cursor <cursoragent@cursor.com>
</commit_message>
<xml_diff>
--- a/Scram Book/Explorer Tab/Rovvy_Explorer_Scrum_Book.xlsx
+++ b/Scram Book/Explorer Tab/Rovvy_Explorer_Scrum_Book.xlsx
@@ -1346,14 +1346,14 @@
           <t>Visual</t>
         </is>
       </c>
-      <c r="C20" s="20" t="inlineStr">
-        <is>
-          <t>[2026-10-09] Map crop fallback at z17 (no stock images)</t>
+      <c r="C20" s="19" t="inlineStr">
+        <is>
+          <t>[2026-10-09] map crop deferred: server-side pre-render (R2) planned</t>
         </is>
       </c>
       <c r="D20" s="20" t="inlineStr">
         <is>
-          <t>Complete in code</t>
+          <t>Partial</t>
         </is>
       </c>
       <c r="E20" s="13" t="inlineStr">
@@ -1373,7 +1373,7 @@
       </c>
       <c r="H20" s="13" t="inlineStr">
         <is>
-          <t>2026-10-09: place-panel-map-tile via explore-listing-media; Map preview label; drawer + cards. User review 2026-09-22; Audit IDs 31,47</t>
+          <t>2026-10-09: Removed live feed MapLibre crops (ExploreMapCrop); compact text cards; drawer map only. Vitest explore suite. 2026-10-09: place-panel-map-tile via explore-listing-media; Map preview label; drawer + cards. User review 2026-09-22; Audit IDs 31,47</t>
         </is>
       </c>
       <c r="I20" s="13" t="inlineStr">
@@ -5129,7 +5129,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:N103"/>
+  <dimension ref="A1:N104"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="18" customWidth="1" min="1" max="1"/>
@@ -11650,6 +11650,28 @@
         </is>
       </c>
     </row>
+    <row r="104">
+      <c r="A104" t="inlineStr">
+        <is>
+          <t>2026-10-09 04:12</t>
+        </is>
+      </c>
+      <c r="B104" t="inlineStr">
+        <is>
+          <t>G12</t>
+        </is>
+      </c>
+      <c r="C104" t="inlineStr">
+        <is>
+          <t>Feed map crop removed; G12 Partial</t>
+        </is>
+      </c>
+      <c r="D104" t="inlineStr">
+        <is>
+          <t>2026-10-09: Removed live feed MapLibre crops (ExploreMapCrop); compact text cards; drawer map only. Vitest explore suite.</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>

</xml_diff>

<commit_message>
F47: Wikidata dry-run caches and Ticketmaster venue photo pipeline with spine media priority and pytest.
Co-authored-by: Cursor <cursoragent@cursor.com>
</commit_message>
<xml_diff>
--- a/Scram Book/Explorer Tab/Rovvy_Explorer_Scrum_Book.xlsx
+++ b/Scram Book/Explorer Tab/Rovvy_Explorer_Scrum_Book.xlsx
@@ -4369,7 +4369,7 @@
       </c>
       <c r="C73" s="19" t="inlineStr">
         <is>
-          <t>[2026-10-05] Drawer photo</t>
+          <t>[2026-10-12] F47 Drawer photo (Wikidata + Commons + Ticketmaster venue)</t>
         </is>
       </c>
       <c r="D73" s="19" t="inlineStr">
@@ -4394,7 +4394,7 @@
       </c>
       <c r="H73" s="9" t="inlineStr">
         <is>
-          <t>2026-10-05 Orlando dry-run: scripts/05_enrich_wikidata.py --dry-run --metros orlando → 342 Wikidata entities, 15,372 places, 99 match candidates, 166 rejected, 2 ambiguous (no DB writes). 07_enrich_wikimedia_photos --dry-run --metros orlando → 0 QIDs (no Orlando wikidata_qid rows yet). GET /explore/places Orlando lat/lon 50 rows, 0 image_url until wikidata+photos applied on Postgres. Prod DB write pending operator approval. 2026-10-05: Drawer + cards show Wikimedia Commons photos (259 Chicago places, free licenses only, author + license credit) and approved user uploads (R2, EXIF/GPS stripped, moderated). Coverage is landmarks only (~5 of 96 nearest). | Explore audit ID 47; Drawer displays a detail-photo placeholder rather than listing media.</t>
+          <t>2026-10-12: 05_enrich_wikidata --dry-run --metros milwaukee orlando → milwaukee 317 matches / 9,269 places; orlando 99 / 15,374 (sample 20 printed in dry-run). 07_enrich_wikimedia --dry-run → 0 rows (no wikidata_qid yet). scaper backfill-ticketmaster-venue-photos --dry-run → 52 linked venues, 18 with TM venue images. Code: scaper/venue_place_media.py pipeline sync; explore_place_spine PLACE_MEDIA_PICK_ORDER (rovvy_user &gt; open_license &gt; licensed_partner); pytest test_ticketmaster_venue_media + spine SQL tests. 2026-10-05 Orlando dry-run: scripts/05_enrich_wikidata.py --dry-run --metros orlando → 342 Wikidata entities, 15,372 places, 99 match candidates, 166 rejected, 2 ambiguous (no DB writes). 07_enrich_wikimedia_photos --dry-run --metros orlando → 0 QIDs (no Orlando wikidata_qid rows yet). GET /explore/places Orlando lat/lon 50 rows, 0 image_url until wikidata+photos applied on Postgres. Prod DB write pending operator approval. 2026-10-05: Drawer + cards show Wikimedia Commons photos (259 Chicago places, free licenses only, author + license credit) and approved user uploads (R2, EXIF/GPS stripped, moderated). Coverage is landmarks only (~5 of 96 nearest). | Explore audit ID 47; Drawer displays a detail-photo placeholder rather than listing media.</t>
         </is>
       </c>
       <c r="I73" s="9" t="inlineStr">
@@ -4404,7 +4404,7 @@
       </c>
       <c r="J73" t="inlineStr">
         <is>
-          <t>Cursor: after operator approves prod Postgres, run 05_enrich_wikidata orlando (no --dry-run), then 07_enrich_wikimedia_photos orlando; verify map_spine_row image_url/image_attribution; ExploreDetailDrawer hero image; pytest/vitest if mapper changes.</t>
+          <t>Operator approve prod writes: 05_enrich_wikidata milwaukee orlando; 07_enrich_wikimedia_photos same; scaper backfill-ticketmaster-venue-photos (no --dry-run). Browser QA Milwaukee + Chicago feeds for credits.</t>
         </is>
       </c>
       <c r="K73" t="inlineStr">
@@ -5129,7 +5129,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:N104"/>
+  <dimension ref="A1:N105"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="18" customWidth="1" min="1" max="1"/>
@@ -11672,6 +11672,72 @@
         </is>
       </c>
     </row>
+    <row r="105">
+      <c r="A105" s="16" t="n">
+        <v>46307.35416666666</v>
+      </c>
+      <c r="B105" t="inlineStr">
+        <is>
+          <t>F47</t>
+        </is>
+      </c>
+      <c r="C105" t="inlineStr">
+        <is>
+          <t>Capability</t>
+        </is>
+      </c>
+      <c r="D105" t="inlineStr">
+        <is>
+          <t>[2026-10-12] F47 Drawer photo (Wikidata + Commons + Ticketmaster venue)</t>
+        </is>
+      </c>
+      <c r="E105" t="inlineStr">
+        <is>
+          <t>Partial</t>
+        </is>
+      </c>
+      <c r="F105" t="inlineStr">
+        <is>
+          <t>Later</t>
+        </is>
+      </c>
+      <c r="G105" t="inlineStr">
+        <is>
+          <t>Easy</t>
+        </is>
+      </c>
+      <c r="H105" t="inlineStr">
+        <is>
+          <t>Pass verified image_url + image_attribution on drawer/card for spine places; Orlando metro after wikidata + Commons enrich; broaden beyond Chicago-only.</t>
+        </is>
+      </c>
+      <c r="I105" t="inlineStr">
+        <is>
+          <t>2026-10-12: 05_enrich_wikidata --dry-run --metros milwaukee orlando → milwaukee 317 matches / 9,269 places; orlando 99 / 15,374 (sample 20 printed in dry-run). 07_enrich_wikimedia --dry-run → 0 rows (no wikidata_qid yet). scaper backfill-ticketmaster-venue-photos --dry-run → 52 linked venues, 18 with TM venue images. Code: scaper/venue_place_media.py pipeline sync; explore_place_spine PLACE_MEDIA_PICK_ORDER (rovvy_user &gt; open_license &gt; licensed_partner); pytest test_ticketmaster_venue_media + spine SQL tests. 2026-10-05 Orlando dry-run: scripts/05_enrich_wikidata.py --dry-run --metros orlando → 342 Wikidata entities, 15,372 places, 99 match candidates, 166 rejected, 2 ambiguous (no DB writes). 07_enrich_wikimedia_photos --dry-run --metros orlando → 0 QIDs (no Orlando wikidata_qid rows yet). GET /explore/places Orlando lat/lon 50 rows, 0 image_url until wikidata+photos applied on Postgres. Prod DB write pending operator approval. 2026-10-05: Drawer + cards show Wikimedia Commons photos (259 Chicago places, free licenses only, author + license credit) and approved user uploads (R2, EXIF/GPS stripped, moderated). Coverage is landmarks only (~5 of 96 nearest). | Explore audit ID 47; Drawer displays a detail-photo placeholder rather than listing media.</t>
+        </is>
+      </c>
+      <c r="J105" t="inlineStr">
+        <is>
+          <t>See acceptance / next action</t>
+        </is>
+      </c>
+      <c r="K105" t="inlineStr">
+        <is>
+          <t>Feature</t>
+        </is>
+      </c>
+      <c r="L105" t="inlineStr"/>
+      <c r="M105" t="inlineStr">
+        <is>
+          <t>Operator approve prod writes: 05_enrich_wikidata milwaukee orlando; 07_enrich_wikimedia_photos same; scaper backfill-ticketmaster-venue-photos (no --dry-run). Browser QA Milwaukee + Chicago feeds for credits.</t>
+        </is>
+      </c>
+      <c r="N105" t="inlineStr">
+        <is>
+          <t>Explorer</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>

</xml_diff>

<commit_message>
F27: server-side per-day provider round-robin in the Explore events reader (SQL window before paging)
scaper_events_for_city orders by (local_day, provider_rank_in_day, start_time, id) via row_number() OVER (PARTITION BY local_day, provider) over the shared visibility CTE; total/paging unchanged, generic over providers; explorer_v2 keyset untouched (not used by the Explore hub). Tests: tests/test_explore_provider_mix_pg.py 5/5 on rolled-back Postgres (page-1 mix, day order, single provider, paging exactly-once, 3 providers); SQL-shape unit test; backend 983 passed / 35 skipped. Live read-only: Chicago weekend EB in first 24 2->3 (cards 2/4/6), Orlando 14-day 1->2; Chicago Tonight stays 0 (no Eventbrite rows today by design). Scram Book: F27 row green + Context Log + README entry; workbook backup kept.

Co-authored-by: Cursor <cursoragent@cursor.com>
</commit_message>
<xml_diff>
--- a/Scram Book/Explorer Tab/Rovvy_Explorer_Scrum_Book.xlsx
+++ b/Scram Book/Explorer Tab/Rovvy_Explorer_Scrum_Book.xlsx
@@ -62,7 +62,7 @@
       <sz val="14"/>
     </font>
   </fonts>
-  <fills count="10">
+  <fills count="11">
     <fill>
       <patternFill/>
     </fill>
@@ -109,6 +109,12 @@
         <fgColor rgb="00DDF3E3"/>
       </patternFill>
     </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor rgb="00DDF3E3"/>
+        <bgColor rgb="00DDF3E3"/>
+      </patternFill>
+    </fill>
   </fills>
   <borders count="1">
     <border/>
@@ -116,7 +122,7 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="22">
+  <cellXfs count="23">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="2" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
@@ -141,6 +147,7 @@
     <xf numFmtId="0" fontId="5" fillId="8" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="5" fillId="9" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="0" fillId="9" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="5" fillId="10" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
   </cellXfs>
   <cellStyles count="1">
     <cellStyle name="Normal" xfId="0"/>
@@ -3227,12 +3234,12 @@
           <t>Capability</t>
         </is>
       </c>
-      <c r="C53" s="20" t="inlineStr">
-        <is>
-          <t>[2026-10-09] Mixed provider feed interleave per day</t>
-        </is>
-      </c>
-      <c r="D53" s="20" t="inlineStr">
+      <c r="C53" s="22" t="inlineStr">
+        <is>
+          <t>[2026-10-14] Mixed provider feed: server-side per-day provider round-robin (SQL window, before paging)</t>
+        </is>
+      </c>
+      <c r="D53" s="22" t="inlineStr">
         <is>
           <t>Complete in code</t>
         </is>
@@ -3254,7 +3261,7 @@
       </c>
       <c r="H53" s="9" t="inlineStr">
         <is>
-          <t>2026-10-09: interleaveEventSlotsByDayAndProvider; Eventbrite in first 24 when present. Vitest explore-feed-phase1. 2026-09-23: Client Load more (+24 over bounded fetched pool) ships on main Explore hub (G15). F27 stays Partial: no provider/backend pagination or additional API pages; only in-memory reveal of rows already returned.</t>
+          <t>2026-10-14: scaper_events_for_city (v1 /explore/events reader behind the Explore hub) now orders by (local_day, provider_rank_in_day, start_time, id) with row_number() OVER (PARTITION BY local_day, provider) over the shared visibility CTE, before LIMIT/OFFSET; no Python sort, generic over providers, dedup/visibility CTE untouched; explorer_v2 keyset left as is (serves explore-v2/map only). Tests: tests/test_explore_provider_mix_pg.py 5/5 on rolled-back Supabase (30 TM + 3 EB -&gt; page 1 of 12 has all 3 EB alternating; day 1 before day 2; single provider = start_time; paging 45 rows exactly once; 3-provider round-robin), unit SQL-shape test in test_explore_scaper_events.py; backend 983 passed / 35 skipped. Live read-only (2026-10-14): Chicago 454 visible next 14 d (TM 439 / EB 53 upcoming total; EB 0 today, 1 tomorrow, 3+2 weekend); EB in first 24: Tonight 0-&gt;0 (no EB today, by design nothing jumps ahead of today), Tomorrow 1-&gt;1 (now card #2), This weekend 2-&gt;3 (cards #2/#4/#6), first 100 of 14-day window 1-&gt;2. Orlando 110 visible: Tonight 1-&gt;1 (card #2), Next week 1-&gt;2, 14-day 1-&gt;2. 2026-10-09: interleaveEventSlotsByDayAndProvider; Eventbrite in first 24 when present. Vitest explore-feed-phase1. 2026-09-23: Client Load more (+24 over bounded fetched pool) ships on main Explore hub (G15). F27 stays Partial: no provider/backend pagination or additional API pages; only in-memory reveal of rows already returned.</t>
         </is>
       </c>
       <c r="I53" s="9" t="inlineStr">
@@ -3264,7 +3271,7 @@
       </c>
       <c r="J53" t="inlineStr">
         <is>
-          <t>Cursor: close the gap in evidence (2026-09-23: Client Load more (+24 over bounded fetched pool) ships on main Explore hub (G15). F27 stays Partial: no p...) with minimal diff. Implement acceptance: Mix categories intentionally and connect pagination.. Stack: frontend/app/(dashboard)/explore/* + app/routes/explore.py + app/services/explore_*; add 200/401/422 API tests for new endpoints; no logic in route handlers. Importance=High, difficulty=Easy. fetchExploreHub + classifyExploreSourceLoadState; partial failure copy when one source fails.</t>
+          <t>Cursor: keep ordering key (local_day, provider_rank_in_day, start_time, id); any change to the mix stays in SQL (app/services/explore_scaper_events.py) and must keep total/paging consistent; re-run tests/test_explore_provider_mix_pg.py with SCAPER_PG_TEST_URL.</t>
         </is>
       </c>
       <c r="K53" t="inlineStr">
@@ -4394,7 +4401,7 @@
       </c>
       <c r="H73" s="9" t="inlineStr">
         <is>
-          <t>2026-10-12: 05_enrich_wikidata --dry-run --metros milwaukee orlando → milwaukee 317 matches / 9,269 places; orlando 99 / 15,374 (sample 20 printed in dry-run). 07_enrich_wikimedia --dry-run → 0 rows (no wikidata_qid yet). scaper backfill-ticketmaster-venue-photos --dry-run → 52 linked venues, 18 with TM venue images. Code: scaper/venue_place_media.py pipeline sync; explore_place_spine PLACE_MEDIA_PICK_ORDER (rovvy_user &gt; open_license &gt; licensed_partner); pytest test_ticketmaster_venue_media + spine SQL tests. 2026-10-05 Orlando dry-run: scripts/05_enrich_wikidata.py --dry-run --metros orlando → 342 Wikidata entities, 15,372 places, 99 match candidates, 166 rejected, 2 ambiguous (no DB writes). 07_enrich_wikimedia_photos --dry-run --metros orlando → 0 QIDs (no Orlando wikidata_qid rows yet). GET /explore/places Orlando lat/lon 50 rows, 0 image_url until wikidata+photos applied on Postgres. Prod DB write pending operator approval. 2026-10-05: Drawer + cards show Wikimedia Commons photos (259 Chicago places, free licenses only, author + license credit) and approved user uploads (R2, EXIF/GPS stripped, moderated). Coverage is landmarks only (~5 of 96 nearest). | Explore audit ID 47; Drawer displays a detail-photo placeholder rather than listing media.</t>
+          <t>2026-10-12 APPLY: 05_enrich_wikidata milwaukee orlando → rows_updated 317+99=416 QIDs. 07_enrich_wikimedia → 416 eligible, 197 P18, 196 free-licence Commons → 196 place_media inserted. backfill-ticketmaster-venue-photos → 52 candidates, 18 with venue images, 10 inserted (8 skipped higher-priority). Operator browser QA Milwaukee+Chicago pending. 2026-10-12: 05_enrich_wikidata --dry-run --metros milwaukee orlando → milwaukee 317 matches / 9,269 places; orlando 99 / 15,374 (sample 20 printed in dry-run). 07_enrich_wikimedia --dry-run → 0 rows (no wikidata_qid yet). scaper backfill-ticketmaster-venue-photos --dry-run → 52 linked venues, 18 with TM venue images. Code: scaper/venue_place_media.py pipeline sync; explore_place_spine PLACE_MEDIA_PICK_ORDER (rovvy_user &gt; open_license &gt; licensed_partner); pytest test_ticketmaster_venue_media + spine SQL tests. 2026-10-05 Orlando dry-run: scripts/05_enrich_wikidata.py --dry-run --metros orlando → 342 Wikidata entities, 15,372 places, 99 match candidates, 166 rejected, 2 ambiguous (no DB writes). 07_enrich_wikimedia_photos --dry-run --metros orlando → 0 QIDs (no Orlando wikidata_qid rows yet). GET /explore/places Orlando lat/lon 50 rows, 0 image_url until wikidata+photos applied on Postgres. Prod DB write pending operator approval. 2026-10-05: Drawer + cards show Wikimedia Commons photos (259 Chicago places, free licenses only, author + license credit) and approved user uploads (R2, EXIF/GPS stripped, moderated). Coverage is landmarks only (~5 of 96 nearest). | Explore audit ID 47; Drawer displays a detail-photo placeholder rather than listing media.</t>
         </is>
       </c>
       <c r="I73" s="9" t="inlineStr">
@@ -5129,7 +5136,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:N105"/>
+  <dimension ref="A1:N107"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="18" customWidth="1" min="1" max="1"/>
@@ -11726,13 +11733,137 @@
           <t>Feature</t>
         </is>
       </c>
-      <c r="L105" t="inlineStr"/>
       <c r="M105" t="inlineStr">
         <is>
           <t>Operator approve prod writes: 05_enrich_wikidata milwaukee orlando; 07_enrich_wikimedia_photos same; scaper backfill-ticketmaster-venue-photos (no --dry-run). Browser QA Milwaukee + Chicago feeds for credits.</t>
         </is>
       </c>
       <c r="N105" t="inlineStr">
+        <is>
+          <t>Explorer</t>
+        </is>
+      </c>
+    </row>
+    <row r="106">
+      <c r="A106" s="16" t="n">
+        <v>46307.375</v>
+      </c>
+      <c r="B106" t="inlineStr">
+        <is>
+          <t>F47</t>
+        </is>
+      </c>
+      <c r="C106" t="inlineStr">
+        <is>
+          <t>Capability</t>
+        </is>
+      </c>
+      <c r="D106" t="inlineStr">
+        <is>
+          <t>[2026-10-12] F47 Drawer photo (Wikidata + Commons + Ticketmaster venue)</t>
+        </is>
+      </c>
+      <c r="E106" t="inlineStr">
+        <is>
+          <t>Partial</t>
+        </is>
+      </c>
+      <c r="F106" t="inlineStr">
+        <is>
+          <t>Later</t>
+        </is>
+      </c>
+      <c r="G106" t="inlineStr">
+        <is>
+          <t>Easy</t>
+        </is>
+      </c>
+      <c r="H106" t="inlineStr">
+        <is>
+          <t>Pass verified image_url + image_attribution on drawer/card for spine places; Orlando metro after wikidata + Commons enrich; broaden beyond Chicago-only.</t>
+        </is>
+      </c>
+      <c r="I106" t="inlineStr">
+        <is>
+          <t>2026-10-12 APPLY: 05_enrich_wikidata milwaukee orlando → rows_updated 317+99=416 QIDs. 07_enrich_wikimedia → 416 eligible, 197 P18, 196 free-licence Commons → 196 place_media inserted. backfill-ticketmaster-venue-photos → 52 candidates, 18 with venue images, 10 inserted (8 skipped higher-priority). Operator browser QA Milwaukee+Chicago pending. 2026-10-12: 05_enrich_wikidata --dry-run --metros milwaukee orlando → milwaukee 317 matches / 9,269 places; orlando 99 / 15,374 (sample 20 printed in dry-run). 07_enrich_wikimedia --dry-run → 0 rows (no wikidata_qid yet). scaper backfill-ticketmaster-venue-photos --dry-run → 52 linked venues, 18 with TM venue images. Code: scaper/venue_place_media.py pipeline sync; explore_place_spine PLACE_MEDIA_PICK_ORDER (rovvy_user &gt; open_license &gt; licensed_partner); pytest test_ticketmaster_venue_media + spine SQL tests. 2026-10-05 Orlando dry-run: scripts/05_enrich_wikidata.py --dry-run --metros orlando → 342 Wikidata entities, 15,372 places, 99 match candidates, 166 rejected, 2 ambiguous (no DB writes). 07_enrich_wikimedia_photos --dry-run --metros orlando → 0 QIDs (no Orlando wikidata_qid rows yet). GET /explore/places Orlando lat/lon 50 rows, 0 image_url until wikidata+photos applied on Postgres. Prod DB write pending operator approval. 2026-10-05: Drawer + cards show Wikimedia Commons photos (259 Chicago places, free licenses only, author + license credit) and approved user uploads (R2, EXIF/GPS stripped, moderated). Coverage is landmarks only (~5 of 96 nearest). | Explore audit ID 47; Drawer displays a detail-photo placeholder rather than listing media.</t>
+        </is>
+      </c>
+      <c r="K106" t="inlineStr">
+        <is>
+          <t>Feature</t>
+        </is>
+      </c>
+      <c r="M106" t="inlineStr">
+        <is>
+          <t>Operator approve prod writes: 05_enrich_wikidata milwaukee orlando; 07_enrich_wikimedia_photos same; scaper backfill-ticketmaster-venue-photos (no --dry-run). Browser QA Milwaukee + Chicago feeds for credits.</t>
+        </is>
+      </c>
+      <c r="N106" t="inlineStr">
+        <is>
+          <t>Explorer</t>
+        </is>
+      </c>
+    </row>
+    <row r="107">
+      <c r="A107" s="16" t="n">
+        <v>46309.14236111111</v>
+      </c>
+      <c r="B107" t="inlineStr">
+        <is>
+          <t>F27</t>
+        </is>
+      </c>
+      <c r="C107" t="inlineStr">
+        <is>
+          <t>Capability</t>
+        </is>
+      </c>
+      <c r="D107" t="inlineStr">
+        <is>
+          <t>[2026-10-14] Mixed provider feed: server-side per-day provider round-robin (SQL window, before paging)</t>
+        </is>
+      </c>
+      <c r="E107" t="inlineStr">
+        <is>
+          <t>Complete in code</t>
+        </is>
+      </c>
+      <c r="F107" t="inlineStr">
+        <is>
+          <t>High</t>
+        </is>
+      </c>
+      <c r="G107" t="inlineStr">
+        <is>
+          <t>Easy</t>
+        </is>
+      </c>
+      <c r="H107" t="inlineStr">
+        <is>
+          <t>Mix categories intentionally and connect pagination.</t>
+        </is>
+      </c>
+      <c r="I107" t="inlineStr">
+        <is>
+          <t>2026-10-14: scaper_events_for_city (v1 /explore/events reader behind the Explore hub) now orders by (local_day, provider_rank_in_day, start_time, id) with row_number() OVER (PARTITION BY local_day, provider) over the shared visibility CTE, before LIMIT/OFFSET; no Python sort, generic over providers, dedup/visibility CTE untouched; explorer_v2 keyset left as is (serves explore-v2/map only). Tests: tests/test_explore_provider_mix_pg.py 5/5 on rolled-back Supabase (30 TM + 3 EB -&gt; page 1 of 12 has all 3 EB alternating; day 1 before day 2; single provider = start_time; paging 45 rows exactly once; 3-provider round-robin), unit SQL-shape test in test_explore_scaper_events.py; backend 983 passed / 35 skipped. Live read-only (2026-10-14): Chicago 454 visible next 14 d (TM 439 / EB 53 upcoming total; EB 0 today, 1 tomorrow, 3+2 weekend); EB in first 24: Tonight 0-&gt;0 (no EB today, by design nothing jumps ahead of today), Tomorrow 1-&gt;1 (now card #2), This weekend 2-&gt;3 (cards #2/#4/#6), first 100 of 14-day window 1-&gt;2. Orlando 110 visible: Tonight 1-&gt;1 (card #2), Next week 1-&gt;2, 14-day 1-&gt;2.</t>
+        </is>
+      </c>
+      <c r="J107" t="inlineStr">
+        <is>
+          <t>Browser QA /explore</t>
+        </is>
+      </c>
+      <c r="K107" t="inlineStr">
+        <is>
+          <t>Feature</t>
+        </is>
+      </c>
+      <c r="M107" t="inlineStr">
+        <is>
+          <t>Browser QA /explore Chicago 'This weekend' (Eventbrite at cards 2/4/6). If the owner wants Eventbrite on days with 0 EB rows, that is a different rule (cross-day lift) and needs a decision.</t>
+        </is>
+      </c>
+      <c r="N107" t="inlineStr">
         <is>
           <t>Explorer</t>
         </is>

</xml_diff>

<commit_message>
F27b provider mix across the window + F50 place facts (Wikipedia/OSM, migration not applied)
F27b: scaper_events_for_city reserves a minimum share (1 in 6) for non-dominant providers across the whole window via a window-function mix_position, before LIMIT/OFFSET. Fixed AmbiguousColumn SQL bug found in review. Live read-only: Chicago/Orlando page 1 and 2 show 1 Eventbrite per 7 cards; totals unchanged (492/137). Postgres suites 28 passed, backend 998 passed at that point.

F50: place_facts table migration 012 (not applied), Wikipedia/Wikidata and OSM fact services, grid-indexed OSM matching, facts on the place spine endpoint, drawer display with credits, /legal/data entries. Tests: test_place_facts 12+, spine 7, frontend facts 4. Dry-run default; no production write.

Scram Book: workbook rows and README entries.

Co-Authored-By: Claude Sonnet 5.5 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/Scram Book/Explorer Tab/Rovvy_Explorer_Scrum_Book.xlsx
+++ b/Scram Book/Explorer Tab/Rovvy_Explorer_Scrum_Book.xlsx
@@ -505,7 +505,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A2:K85"/>
+  <dimension ref="A2:K87"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="9" customWidth="1" min="1" max="1"/>
@@ -3234,12 +3234,12 @@
           <t>Capability</t>
         </is>
       </c>
-      <c r="C53" s="22" t="inlineStr">
-        <is>
-          <t>[2026-10-14] Mixed provider feed: server-side per-day provider round-robin (SQL window, before paging)</t>
-        </is>
-      </c>
-      <c r="D53" s="22" t="inlineStr">
+      <c r="C53" s="20" t="inlineStr">
+        <is>
+          <t>[2026-10-14] F27b Mixed provider feed: window-wide share (MIN_PROVIDER_SHARE_EVERY=6)</t>
+        </is>
+      </c>
+      <c r="D53" s="19" t="inlineStr">
         <is>
           <t>Complete in code</t>
         </is>
@@ -3261,7 +3261,7 @@
       </c>
       <c r="H53" s="9" t="inlineStr">
         <is>
-          <t>2026-10-14: scaper_events_for_city (v1 /explore/events reader behind the Explore hub) now orders by (local_day, provider_rank_in_day, start_time, id) with row_number() OVER (PARTITION BY local_day, provider) over the shared visibility CTE, before LIMIT/OFFSET; no Python sort, generic over providers, dedup/visibility CTE untouched; explorer_v2 keyset left as is (serves explore-v2/map only). Tests: tests/test_explore_provider_mix_pg.py 5/5 on rolled-back Supabase (30 TM + 3 EB -&gt; page 1 of 12 has all 3 EB alternating; day 1 before day 2; single provider = start_time; paging 45 rows exactly once; 3-provider round-robin), unit SQL-shape test in test_explore_scaper_events.py; backend 983 passed / 35 skipped. Live read-only (2026-10-14): Chicago 454 visible next 14 d (TM 439 / EB 53 upcoming total; EB 0 today, 1 tomorrow, 3+2 weekend); EB in first 24: Tonight 0-&gt;0 (no EB today, by design nothing jumps ahead of today), Tomorrow 1-&gt;1 (now card #2), This weekend 2-&gt;3 (cards #2/#4/#6), first 100 of 14-day window 1-&gt;2. Orlando 110 visible: Tonight 1-&gt;1 (card #2), Next week 1-&gt;2, 14-day 1-&gt;2. 2026-10-09: interleaveEventSlotsByDayAndProvider; Eventbrite in first 24 when present. Vitest explore-feed-phase1. 2026-09-23: Client Load more (+24 over bounded fetched pool) ships on main Explore hub (G15). F27 stays Partial: no provider/backend pagination or additional API pages; only in-memory reveal of rows already returned.</t>
+          <t>2026-10-14 (Claude review): fixed AmbiguousColumn bug in the F27b SQL (mixed.* selected mix_position twice; live reader errored on Postgres). After fix: PG suites 27 passed on real Postgres; full backend 997 passed/36 skipped; live read-only: Chicago page1 TTTTTTETTTTTTETTTTTTETTT, page2 TTTETTTTTTETTTTTTETTTTTT (1 Eventbrite in every 7), Orlando same pattern; total unchanged (Chicago 492, Orlando 137). 2026-10-14 F27b: explore_scaper_events mix_position across full date window (dominant provider rank_p; others rank_p*6); ORDER BY mix_position,start_time,id. tests/test_explore_provider_mix_pg.py rewritten (5 cases); test_explore_scaper_events SQL shape updated. pytest test_place_facts OSM grid 2 new + test_explore_scaper_events 1 passed; PG mix 5 skipped without SCAPER_PG_TEST_URL. Live Chicago/Orlando first-24 EB counts: not run (DATABASE_URL unset in verify script). 2026-10-14: scaper_events_for_city (v1 /explore/events reader behind the Explore hub) now orders by (local_day, provider_rank_in_day, start_time, id) with row_number() OVER (PARTITION BY local_day, provider) over the shared visibility CTE, before LIMIT/OFFSET; no Python sort, generic over providers, dedup/visibility CTE untouched; explorer_v2 keyset left as is (serves explore-v2/map only). Tests: tests/test_explore_provider_mix_pg.py 5/5 on rolled-back Supabase (30 TM + 3 EB -&gt; page 1 of 12 has all 3 EB alternating; day 1 before day 2; single provider = start_time; paging 45 rows exactly once; 3-provider round-robin), unit SQL-shape test in test_explore_scaper_events.py; backend 983 passed / 35 skipped. Live read-only (2026-10-14): Chicago 454 visible next 14 d (TM 439 / EB 53 upcoming total; EB 0 today, 1 tomorrow, 3+2 weekend); EB in first 24: Tonight 0-&gt;0 (no EB today, by design nothing jumps ahead of today), Tomorrow 1-&gt;1 (now card #2), This weekend 2-&gt;3 (cards #2/#4/#6), first 100 of 14-day window 1-&gt;2. Orlando 110 visible: Tonight 1-&gt;1 (card #2), Next week 1-&gt;2, 14-day 1-&gt;2. 2026-10-09: interleaveEventSlotsByDayAndProvider; Eventbrite in first 24 when present. Vitest explore-feed-phase1. 2026-09-23: Client Load more (+24 over bounded fetched pool) ships on main Explore hub (G15). F27 stays Partial: no provider/backend pagination or additional API pages; only in-memory reveal of rows already returned.</t>
         </is>
       </c>
       <c r="I53" s="9" t="inlineStr">
@@ -3271,7 +3271,7 @@
       </c>
       <c r="J53" t="inlineStr">
         <is>
-          <t>Cursor: keep ordering key (local_day, provider_rank_in_day, start_time, id); any change to the mix stays in SQL (app/services/explore_scaper_events.py) and must keep total/paging consistent; re-run tests/test_explore_provider_mix_pg.py with SCAPER_PG_TEST_URL.</t>
+          <t>Deploy (push) so production serves it; owner decision pending on push.</t>
         </is>
       </c>
       <c r="K53" t="inlineStr">
@@ -5096,6 +5096,55 @@
       <c r="J85" t="inlineStr">
         <is>
           <t>Owner: apply migration 011; set CONTACT_EMAIL if switching off rovvy230@gmail.com</t>
+        </is>
+      </c>
+    </row>
+    <row r="86">
+      <c r="A86" s="21" t="inlineStr">
+        <is>
+          <t>F50b</t>
+        </is>
+      </c>
+      <c r="C86" s="21" t="inlineStr">
+        <is>
+          <t>[2026-10-14] Place facts: Wikipedia + OSM hours (Chicago pilot; spec F50)</t>
+        </is>
+      </c>
+      <c r="D86" s="21" t="inlineStr">
+        <is>
+          <t>Complete in code</t>
+        </is>
+      </c>
+      <c r="H86" s="21" t="inlineStr">
+        <is>
+          <t>2026-10-14: migrations/012_place_facts.sql (not applied); scripts/12_fetch_place_facts.py --dry-run; GET /places/spine/{gers_id} facts[]; Explore drawer + /legal/data; pytest test_place_facts 12 passed 1 skipped; vitest explore-place-spine-facts 4 passed.</t>
+        </is>
+      </c>
+      <c r="J86" t="inlineStr">
+        <is>
+          <t>Owner: apply 012 migration; Chicago --write with Geofabrik PBF; report match rate.</t>
+        </is>
+      </c>
+    </row>
+    <row r="87">
+      <c r="A87" s="21" t="inlineStr">
+        <is>
+          <t>F27c</t>
+        </is>
+      </c>
+      <c r="C87" s="21" t="inlineStr">
+        <is>
+          <t>[2026-10-14] Explore TS fixes + provider-mix SQL guard (PhotoTheme, MapLibre zIndex, pytest)</t>
+        </is>
+      </c>
+      <c r="D87" s="21" t="inlineStr">
+        <is>
+          <t>Complete in code</t>
+        </is>
+      </c>
+      <c r="H87" s="21" t="inlineStr">
+        <is>
+          <t>2026-10-14: npx tsc --noEmit 0 errors (was 4: PhotoTheme, nightlife branch, zIndexOffset). vitest 616/616 passed; pytest sqlite CI 998 passed 36 skipped; test_provider_mix_ranked_sql_no_duplicate_rank_columns + pg run notes in test_explore_provider_mix_pg.py / test_place_facts.py.</t>
         </is>
       </c>
     </row>
@@ -5136,7 +5185,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:N107"/>
+  <dimension ref="A1:N111"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="18" customWidth="1" min="1" max="1"/>
@@ -11869,6 +11918,197 @@
         </is>
       </c>
     </row>
+    <row r="108">
+      <c r="A108" s="16" t="n">
+        <v>46309.14583333334</v>
+      </c>
+      <c r="B108" t="inlineStr">
+        <is>
+          <t>F50-place-facts</t>
+        </is>
+      </c>
+      <c r="C108" t="inlineStr">
+        <is>
+          <t>Capability</t>
+        </is>
+      </c>
+      <c r="D108" t="inlineStr">
+        <is>
+          <t>[2026-10-14] Place facts: Wikipedia + OSM hours (Chicago pilot; spec F50)</t>
+        </is>
+      </c>
+      <c r="E108" t="inlineStr">
+        <is>
+          <t>Complete in code</t>
+        </is>
+      </c>
+      <c r="F108" t="inlineStr">
+        <is>
+          <t>Later</t>
+        </is>
+      </c>
+      <c r="G108" t="inlineStr">
+        <is>
+          <t>Easy</t>
+        </is>
+      </c>
+      <c r="I108" t="inlineStr">
+        <is>
+          <t>2026-10-14: migrations/012_place_facts.sql (not applied); scripts/12_fetch_place_facts.py --dry-run; GET /places/spine/{gers_id} facts[]; Explore drawer + /legal/data; pytest test_place_facts 12 passed 1 skipped; vitest explore-place-spine-facts 4 passed.</t>
+        </is>
+      </c>
+      <c r="J108" t="inlineStr">
+        <is>
+          <t>Migration not applied</t>
+        </is>
+      </c>
+      <c r="K108" t="inlineStr">
+        <is>
+          <t>Feature</t>
+        </is>
+      </c>
+      <c r="M108" t="inlineStr">
+        <is>
+          <t>Owner: apply 012 migration; Chicago --write with Geofabrik PBF; report match rate.</t>
+        </is>
+      </c>
+      <c r="N108" t="inlineStr">
+        <is>
+          <t>Explorer</t>
+        </is>
+      </c>
+    </row>
+    <row r="109">
+      <c r="A109" s="16" t="n">
+        <v>46309.15625</v>
+      </c>
+      <c r="B109" t="inlineStr">
+        <is>
+          <t>F27b</t>
+        </is>
+      </c>
+      <c r="C109" t="inlineStr">
+        <is>
+          <t>Capability</t>
+        </is>
+      </c>
+      <c r="D109" t="inlineStr">
+        <is>
+          <t>[2026-10-14] F27b Mixed provider feed: window-wide share (MIN_PROVIDER_SHARE_EVERY=6)</t>
+        </is>
+      </c>
+      <c r="E109" t="inlineStr">
+        <is>
+          <t>Partial</t>
+        </is>
+      </c>
+      <c r="F109" t="inlineStr">
+        <is>
+          <t>Later</t>
+        </is>
+      </c>
+      <c r="G109" t="inlineStr">
+        <is>
+          <t>Easy</t>
+        </is>
+      </c>
+      <c r="I109" t="inlineStr">
+        <is>
+          <t>2026-10-14 F27b: explore_scaper_events mix_position across full date window (dominant provider rank_p; others rank_p*6); ORDER BY mix_position,start_time,id. tests/test_explore_provider_mix_pg.py rewritten (5 cases); test_explore_scaper_events SQL shape updated. pytest test_place_facts OSM grid 2 new + test_explore_scaper_events 1 passed; PG mix 5 skipped without SCAPER_PG_TEST_URL. Live Chicago/Orlando first-24 EB counts: not run (DATABASE_URL unset in verify script). 2026-10-14: scaper_events_for_city (v1 /explore/events reader behind the Explore hub) now orders by (local_day, provider_rank_in_day, start_time, id) with row_number() OVER (PARTITION BY local_day, provider) over the shared visibility CTE, before LIMIT/OFFSET; no Python sort, generic over providers, dedup/visibility CTE untouched; explorer_v2 keyset left as is (serves explore-v2/map only). Tests: tests/test_explore_provider_mix_pg.py 5/5 on rolled-back Supabase (30 TM + 3 EB -&gt; page 1 of 12 has all 3 EB alternating; day 1 before day 2; single provider = start_time; paging 45 rows exactly once; 3-provider round-robin), unit SQL-shape test in test_explore_scaper_events.py; backend 983 passed / 35 skipped. Live read-only (2026-10-14): Chicago 454 visible next 14 d (TM 439 / EB 53 upcoming total; EB 0 today, 1 tomorrow, 3+2 weekend); EB in first 24: Tonight 0-&gt;0 (no EB today, by design nothing jumps ahead of today), Tomorrow 1-&gt;1 (now card #2), This weekend 2-&gt;3 (cards #2/#4/#6), first 100 of 14-day window 1-&gt;2. Orlando 110 visible: Tonight 1-&gt;1 (card #2), Next week 1-&gt;2, 14-day 1-&gt;2. 2026-10-09: interleaveEventSlotsByDayAndProvider; Eventbrite in first 24 when present. Vitest explore-feed-phase1. 2026-09-23: Client Load more (+24 over bounded fetched pool) ships on main Explore hub (G15). F27 stays Partial: no provider/backend pagination or additional API pages; only in-memory reveal of rows already returned.</t>
+        </is>
+      </c>
+      <c r="J109" t="inlineStr">
+        <is>
+          <t>Live EB first-24 pending</t>
+        </is>
+      </c>
+      <c r="K109" t="inlineStr">
+        <is>
+          <t>Feature</t>
+        </is>
+      </c>
+      <c r="M109" t="inlineStr">
+        <is>
+          <t>Run verify_f27_provider_mix_live.py with DATABASE_URL; expect EB&gt;=3 in Chicago first 24 after deploy.</t>
+        </is>
+      </c>
+      <c r="N109" t="inlineStr">
+        <is>
+          <t>Explorer</t>
+        </is>
+      </c>
+    </row>
+    <row r="110">
+      <c r="B110" t="inlineStr">
+        <is>
+          <t>F27b</t>
+        </is>
+      </c>
+      <c r="D110" t="inlineStr">
+        <is>
+          <t>[2026-10-14] F27b Mixed provider feed: window-wide share (verified)</t>
+        </is>
+      </c>
+      <c r="I110" t="inlineStr">
+        <is>
+          <t>2026-10-14 Claude review: fixed AmbiguousColumn SQL bug; PG 27 passed; backend 997 passed; live Chicago/Orlando 1 Eventbrite per 7 cards.</t>
+        </is>
+      </c>
+    </row>
+    <row r="111">
+      <c r="A111" s="16" t="n">
+        <v>46309.15833333333</v>
+      </c>
+      <c r="B111" t="inlineStr">
+        <is>
+          <t>F27c</t>
+        </is>
+      </c>
+      <c r="C111" t="inlineStr">
+        <is>
+          <t>Quality</t>
+        </is>
+      </c>
+      <c r="D111" t="inlineStr">
+        <is>
+          <t>[2026-10-14] Explore TS fixes + provider-mix SQL guard (PhotoTheme, MapLibre zIndex, pytest)</t>
+        </is>
+      </c>
+      <c r="E111" t="inlineStr">
+        <is>
+          <t>Complete in code</t>
+        </is>
+      </c>
+      <c r="F111" t="inlineStr">
+        <is>
+          <t>Later</t>
+        </is>
+      </c>
+      <c r="G111" t="inlineStr">
+        <is>
+          <t>Easy</t>
+        </is>
+      </c>
+      <c r="H111" t="inlineStr"/>
+      <c r="I111" t="inlineStr">
+        <is>
+          <t>2026-10-14: npx tsc --noEmit 0 errors (was 4: PhotoTheme, nightlife branch, zIndexOffset). vitest 616/616 passed; pytest sqlite CI 998 passed 36 skipped; test_provider_mix_ranked_sql_no_duplicate_rank_columns + pg run notes in test_explore_provider_mix_pg.py / test_place_facts.py.</t>
+        </is>
+      </c>
+      <c r="J111" t="inlineStr"/>
+      <c r="K111" t="inlineStr">
+        <is>
+          <t>Feature</t>
+        </is>
+      </c>
+      <c r="L111" t="inlineStr"/>
+      <c r="M111" t="inlineStr"/>
+      <c r="N111" t="inlineStr">
+        <is>
+          <t>Explorer</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>

</xml_diff>

<commit_message>
Scram Book: place-facts spec, F27b/F27c/F50 and flight-removal records
Co-Authored-By: Claude Sonnet 5.5 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/Scram Book/Explorer Tab/Rovvy_Explorer_Scrum_Book.xlsx
+++ b/Scram Book/Explorer Tab/Rovvy_Explorer_Scrum_Book.xlsx
@@ -5185,7 +5185,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:N111"/>
+  <dimension ref="A1:N113"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="18" customWidth="1" min="1" max="1"/>
@@ -12089,23 +12089,53 @@
           <t>Easy</t>
         </is>
       </c>
-      <c r="H111" t="inlineStr"/>
       <c r="I111" t="inlineStr">
         <is>
           <t>2026-10-14: npx tsc --noEmit 0 errors (was 4: PhotoTheme, nightlife branch, zIndexOffset). vitest 616/616 passed; pytest sqlite CI 998 passed 36 skipped; test_provider_mix_ranked_sql_no_duplicate_rank_columns + pg run notes in test_explore_provider_mix_pg.py / test_place_facts.py.</t>
         </is>
       </c>
-      <c r="J111" t="inlineStr"/>
       <c r="K111" t="inlineStr">
         <is>
           <t>Feature</t>
         </is>
       </c>
-      <c r="L111" t="inlineStr"/>
-      <c r="M111" t="inlineStr"/>
       <c r="N111" t="inlineStr">
         <is>
           <t>Explorer</t>
+        </is>
+      </c>
+    </row>
+    <row r="112">
+      <c r="A112" t="inlineStr">
+        <is>
+          <t>2026-10-14</t>
+        </is>
+      </c>
+      <c r="B112" t="inlineStr">
+        <is>
+          <t>Flight product removal (nav/shell)</t>
+        </is>
+      </c>
+      <c r="C112" t="inlineStr">
+        <is>
+          <t>Removed /flights from dashboard nav; Travel README 2026-10-14; pytest 988, vitest 549, tsc clean.</t>
+        </is>
+      </c>
+    </row>
+    <row r="113">
+      <c r="A113" t="inlineStr">
+        <is>
+          <t>2026-10-14</t>
+        </is>
+      </c>
+      <c r="B113" t="inlineStr">
+        <is>
+          <t>Ground-only route intelligence</t>
+        </is>
+      </c>
+      <c r="C113" t="inlineStr">
+        <is>
+          <t>No flight segments in route intelligence; Wayra/copy scrub; pytest 987 vitest 549 tsc clean.</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
Scram Book workbooks: F50b corrected to Partial, F27b live evidence, misaligned log/backlog rows fixed
Co-Authored-By: Claude Sonnet 5.5 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/Scram Book/Explorer Tab/Rovvy_Explorer_Scrum_Book.xlsx
+++ b/Scram Book/Explorer Tab/Rovvy_Explorer_Scrum_Book.xlsx
@@ -122,7 +122,7 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="23">
+  <cellXfs count="24">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="2" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
@@ -148,6 +148,7 @@
     <xf numFmtId="0" fontId="5" fillId="9" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="0" fillId="9" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="5" fillId="10" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="0" fillId="8" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
   </cellXfs>
   <cellStyles count="1">
     <cellStyle name="Normal" xfId="0"/>
@@ -3261,7 +3262,7 @@
       </c>
       <c r="H53" s="9" t="inlineStr">
         <is>
-          <t>2026-10-14 (Claude review): fixed AmbiguousColumn bug in the F27b SQL (mixed.* selected mix_position twice; live reader errored on Postgres). After fix: PG suites 27 passed on real Postgres; full backend 997 passed/36 skipped; live read-only: Chicago page1 TTTTTTETTTTTTETTTTTTETTT, page2 TTTETTTTTTETTTTTTETTTTTT (1 Eventbrite in every 7), Orlando same pattern; total unchanged (Chicago 492, Orlando 137). 2026-10-14 F27b: explore_scaper_events mix_position across full date window (dominant provider rank_p; others rank_p*6); ORDER BY mix_position,start_time,id. tests/test_explore_provider_mix_pg.py rewritten (5 cases); test_explore_scaper_events SQL shape updated. pytest test_place_facts OSM grid 2 new + test_explore_scaper_events 1 passed; PG mix 5 skipped without SCAPER_PG_TEST_URL. Live Chicago/Orlando first-24 EB counts: not run (DATABASE_URL unset in verify script). 2026-10-14: scaper_events_for_city (v1 /explore/events reader behind the Explore hub) now orders by (local_day, provider_rank_in_day, start_time, id) with row_number() OVER (PARTITION BY local_day, provider) over the shared visibility CTE, before LIMIT/OFFSET; no Python sort, generic over providers, dedup/visibility CTE untouched; explorer_v2 keyset left as is (serves explore-v2/map only). Tests: tests/test_explore_provider_mix_pg.py 5/5 on rolled-back Supabase (30 TM + 3 EB -&gt; page 1 of 12 has all 3 EB alternating; day 1 before day 2; single provider = start_time; paging 45 rows exactly once; 3-provider round-robin), unit SQL-shape test in test_explore_scaper_events.py; backend 983 passed / 35 skipped. Live read-only (2026-10-14): Chicago 454 visible next 14 d (TM 439 / EB 53 upcoming total; EB 0 today, 1 tomorrow, 3+2 weekend); EB in first 24: Tonight 0-&gt;0 (no EB today, by design nothing jumps ahead of today), Tomorrow 1-&gt;1 (now card #2), This weekend 2-&gt;3 (cards #2/#4/#6), first 100 of 14-day window 1-&gt;2. Orlando 110 visible: Tonight 1-&gt;1 (card #2), Next week 1-&gt;2, 14-day 1-&gt;2. 2026-10-09: interleaveEventSlotsByDayAndProvider; Eventbrite in first 24 when present. Vitest explore-feed-phase1. 2026-09-23: Client Load more (+24 over bounded fetched pool) ships on main Explore hub (G15). F27 stays Partial: no provider/backend pagination or additional API pages; only in-memory reveal of rows already returned.</t>
+          <t>2026-10-15: pushed 7e7c8d2, CI test+deploy green; LIVE API Chicago first 24 = TTTTTETTTTTTTETTTTTTETTT (3 Eventbrite), total 489. 2026-10-14 (Claude review): fixed AmbiguousColumn bug in the F27b SQL (mixed.* selected mix_position twice; live reader errored on Postgres). After fix: PG suites 27 passed on real Postgres; full backend 997 passed/36 skipped; live read-only: Chicago page1 TTTTTTETTTTTTETTTTTTETTT, page2 TTTETTTTTTETTTTTTETTTTTT (1 Eventbrite in every 7), Orlando same pattern; total unchanged (Chicago 492, Orlando 137). 2026-10-14 F27b: explore_scaper_events mix_position across full date window (dominant provider rank_p; others rank_p*6); ORDER BY mix_position,start_time,id. tests/test_explore_provider_mix_pg.py rewritten (5 cases); test_explore_scaper_events SQL shape updated. pytest test_place_facts OSM grid 2 new + test_explore_scaper_events 1 passed; PG mix 5 skipped without SCAPER_PG_TEST_URL. Live Chicago/Orlando first-24 EB counts: not run (DATABASE_URL unset in verify script). 2026-10-14: scaper_events_for_city (v1 /explore/events reader behind the Explore hub) now orders by (local_day, provider_rank_in_day, start_time, id) with row_number() OVER (PARTITION BY local_day, provider) over the shared visibility CTE, before LIMIT/OFFSET; no Python sort, generic over providers, dedup/visibility CTE untouched; explorer_v2 keyset left as is (serves explore-v2/map only). Tests: tests/test_explore_provider_mix_pg.py 5/5 on rolled-back Supabase (30 TM + 3 EB -&gt; page 1 of 12 has all 3 EB alternating; day 1 before day 2; single provider = start_time; paging 45 rows exactly once; 3-provider round-robin), unit SQL-shape test in test_explore_scaper_events.py; backend 983 passed / 35 skipped. Live read-only (2026-10-14): Chicago 454 visible next 14 d (TM 439 / EB 53 upcoming total; EB 0 today, 1 tomorrow, 3+2 weekend); EB in first 24: Tonight 0-&gt;0 (no EB today, by design nothing jumps ahead of today), Tomorrow 1-&gt;1 (now card #2), This weekend 2-&gt;3 (cards #2/#4/#6), first 100 of 14-day window 1-&gt;2. Orlando 110 visible: Tonight 1-&gt;1 (card #2), Next week 1-&gt;2, 14-day 1-&gt;2. 2026-10-09: interleaveEventSlotsByDayAndProvider; Eventbrite in first 24 when present. Vitest explore-feed-phase1. 2026-09-23: Client Load more (+24 over bounded fetched pool) ships on main Explore hub (G15). F27 stays Partial: no provider/backend pagination or additional API pages; only in-memory reveal of rows already returned.</t>
         </is>
       </c>
       <c r="I53" s="9" t="inlineStr">
@@ -3271,7 +3272,7 @@
       </c>
       <c r="J53" t="inlineStr">
         <is>
-          <t>Deploy (push) so production serves it; owner decision pending on push.</t>
+          <t>Done in production. Next: more Eventbrite organizers per city (only Chicago/Orlando today).</t>
         </is>
       </c>
       <c r="K53" t="inlineStr">
@@ -5105,24 +5106,24 @@
           <t>F50b</t>
         </is>
       </c>
-      <c r="C86" s="21" t="inlineStr">
+      <c r="C86" s="23" t="inlineStr">
         <is>
           <t>[2026-10-14] Place facts: Wikipedia + OSM hours (Chicago pilot; spec F50)</t>
         </is>
       </c>
       <c r="D86" s="21" t="inlineStr">
         <is>
-          <t>Complete in code</t>
+          <t>Partial</t>
         </is>
       </c>
       <c r="H86" s="21" t="inlineStr">
         <is>
-          <t>2026-10-14: migrations/012_place_facts.sql (not applied); scripts/12_fetch_place_facts.py --dry-run; GET /places/spine/{gers_id} facts[]; Explore drawer + /legal/data; pytest test_place_facts 12 passed 1 skipped; vitest explore-place-spine-facts 4 passed.</t>
+          <t>2026-10-15 status corrected: code reviewed and tests pass, but NOT live. Gaps: migration 012 not applied; Wikipedia dry-run not run (match count unknown); OSM matching not tested on a real Geofabrik PBF; no user-visible effect yet. 2026-10-14: migrations/012_place_facts.sql (not applied); scripts/12_fetch_place_facts.py --dry-run; GET /places/spine/{gers_id} facts[]; Explore drawer + /legal/data; pytest test_place_facts 12 passed 1 skipped; vitest explore-place-spine-facts 4 passed.</t>
         </is>
       </c>
       <c r="J86" t="inlineStr">
         <is>
-          <t>Owner: apply 012 migration; Chicago --write with Geofabrik PBF; report match rate.</t>
+          <t>Next: run Wikipedia dry-run (read-only), then owner applies 012 and approves the Chicago --write; then report match rates (spec 8). Make green only after that.</t>
         </is>
       </c>
     </row>
@@ -5144,7 +5145,7 @@
       </c>
       <c r="H87" s="21" t="inlineStr">
         <is>
-          <t>2026-10-14: npx tsc --noEmit 0 errors (was 4: PhotoTheme, nightlife branch, zIndexOffset). vitest 616/616 passed; pytest sqlite CI 998 passed 36 skipped; test_provider_mix_ranked_sql_no_duplicate_rank_columns + pg run notes in test_explore_provider_mix_pg.py / test_place_facts.py.</t>
+          <t>2026-10-15 note: tsc clean on the full working tree; a clean checkout of HEAD shows 77 tsc errors from other sessions' uncommitted Lounge/Firebase/map-type work (not from F27c). 2026-10-14: npx tsc --noEmit 0 errors (was 4: PhotoTheme, nightlife branch, zIndexOffset). vitest 616/616 passed; pytest sqlite CI 998 passed 36 skipped; test_provider_mix_ranked_sql_no_duplicate_rank_columns + pg run notes in test_explore_provider_mix_pg.py / test_place_facts.py.</t>
         </is>
       </c>
     </row>
@@ -11939,7 +11940,7 @@
       </c>
       <c r="E108" t="inlineStr">
         <is>
-          <t>Complete in code</t>
+          <t>Partial</t>
         </is>
       </c>
       <c r="F108" t="inlineStr">
@@ -12039,14 +12040,29 @@
       </c>
     </row>
     <row r="110">
+      <c r="A110" t="inlineStr">
+        <is>
+          <t>2026-10-14 04:10:00</t>
+        </is>
+      </c>
       <c r="B110" t="inlineStr">
         <is>
           <t>F27b</t>
         </is>
       </c>
+      <c r="C110" t="inlineStr">
+        <is>
+          <t>Quality</t>
+        </is>
+      </c>
       <c r="D110" t="inlineStr">
         <is>
           <t>[2026-10-14] F27b Mixed provider feed: window-wide share (verified)</t>
+        </is>
+      </c>
+      <c r="E110" t="inlineStr">
+        <is>
+          <t>Complete in code</t>
         </is>
       </c>
       <c r="I110" t="inlineStr">
@@ -12113,12 +12129,27 @@
       </c>
       <c r="B112" t="inlineStr">
         <is>
-          <t>Flight product removal (nav/shell)</t>
+          <t>FLIGHT-RM</t>
         </is>
       </c>
       <c r="C112" t="inlineStr">
         <is>
-          <t>Removed /flights from dashboard nav; Travel README 2026-10-14; pytest 988, vitest 549, tsc clean.</t>
+          <t>Removal</t>
+        </is>
+      </c>
+      <c r="D112" t="inlineStr">
+        <is>
+          <t>[2026-10-14] Flight product removed from code + migration 013</t>
+        </is>
+      </c>
+      <c r="E112" t="inlineStr">
+        <is>
+          <t>Complete in code</t>
+        </is>
+      </c>
+      <c r="I112" t="inlineStr">
+        <is>
+          <t>Routes/services/schemas/UI/tests deleted; pushed 7e7c8d2 CI green; migration 013 applied 2026-10-15 (owner, Supabase SQL editor), verified read-only.</t>
         </is>
       </c>
     </row>
@@ -12130,12 +12161,27 @@
       </c>
       <c r="B113" t="inlineStr">
         <is>
-          <t>Ground-only route intelligence</t>
+          <t>ROUTES-GROUND</t>
         </is>
       </c>
       <c r="C113" t="inlineStr">
         <is>
-          <t>No flight segments in route intelligence; Wayra/copy scrub; pytest 987 vitest 549 tsc clean.</t>
+          <t>Capability</t>
+        </is>
+      </c>
+      <c r="D113" t="inlineStr">
+        <is>
+          <t>[2026-10-14] Ground-only route intelligence</t>
+        </is>
+      </c>
+      <c r="E113" t="inlineStr">
+        <is>
+          <t>Complete in code</t>
+        </is>
+      </c>
+      <c r="I113" t="inlineStr">
+        <is>
+          <t>No air segments; long routes return ground_unavailable_reason; Wayra/copy scrubbed; backend 956 passed on a clean checkout.</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
Explore F09: Select-the-date month calendar replaces scrolling day strip
- Remove 14-day calendar strip (and its scroll bar) under the When chips
- Add 'Select the date' chip opening a month calendar: big black date, small
  dark-green event count, month + year nav, past months blocked
- New GET /api/v1/explore/events/calendar: per-day counts via SQL GROUP BY on
  venue-local day over the visibility CTE (no page cap); unsupported city ->
  supported:false, client falls back to its loaded pool
- Picking a day refetches the hub for exactly that day; cards drop the
  'Tonight' label while a calendar day is active
- Verified: pytest 991 passed/36 skipped; Explore vitest 156/30; full vitest
  557/122; tsc 0; browser /explore Oct 23 = 54 (strip showed 1), Nov 14 pick
- Scram Book: Explorer README entry, F09 row Partial (When chips still
  browser-local tz), Cursor Context Log row
</commit_message>
<xml_diff>
--- a/Scram Book/Explorer Tab/Rovvy_Explorer_Scrum_Book.xlsx
+++ b/Scram Book/Explorer Tab/Rovvy_Explorer_Scrum_Book.xlsx
@@ -2209,12 +2209,12 @@
           <t>Capability</t>
         </is>
       </c>
-      <c r="C35" s="9" t="inlineStr">
-        <is>
-          <t>Tonight / Tomorrow / Weekend / Next week</t>
-        </is>
-      </c>
-      <c r="D35" s="9" t="inlineStr">
+      <c r="C35" s="19" t="inlineStr">
+        <is>
+          <t>[2026-10-18] Tonight / Tomorrow / Weekend / Next week + Select-the-date month calendar</t>
+        </is>
+      </c>
+      <c r="D35" s="19" t="inlineStr">
         <is>
           <t>Partial</t>
         </is>
@@ -2231,12 +2231,12 @@
       </c>
       <c r="G35" s="9" t="inlineStr">
         <is>
-          <t>Connect date ranges to queries and use destination timezone.</t>
+          <t>Remaining: compute Tonight/Tomorrow/Weekend/Next week ranges in the destination timezone (calendar day counts already group by venue-local day).</t>
         </is>
       </c>
       <c r="H35" s="9" t="inlineStr">
         <is>
-          <t>2026-09-25: Phase A calendar strip under When row on /explore; days with dated events only; day tap filters feed (events on day + places). Category chips hide at zero. 14-day client fetch widen; no new API. Vitest 107/18. Full month/provider calendar still open.</t>
+          <t>2026-10-18: Scrolling 14-day strip removed. New 'Select the date' chip in the When row opens a month calendar (big black date, small dark-green event count; month + year nav; past months blocked). Counts come from new GET /api/v1/explore/events/calendar (SQL GROUP BY venue-local day over the visibility CTE, no page cap; unsupported city -&gt; supported:false and client counts its loaded pool). Picking a day refetches the hub for exactly that day; cards drop the 'Tonight' label while a day is active. Verified /explore (Hermosa, Chicago): Oct 23 = 54 (strip showed 1), Nov 14 pick -&gt; 3 events + places. pytest 991 passed/36 skipped; Explore Vitest 156/30; full Vitest 557/122; tsc 0. Gap: When-chip ranges still use the browser clock, not destination timezone. 2026-09-25: Phase A calendar strip under When row on /explore; days with dated events only; day tap filters feed (events on day + places). Category chips hide at zero. 14-day client fetch widen; no new API. Vitest 107/18. Full month/provider calendar still open.</t>
         </is>
       </c>
       <c r="I35" s="9" t="inlineStr">
@@ -5186,7 +5186,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:N113"/>
+  <dimension ref="A1:N114"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="18" customWidth="1" min="1" max="1"/>
@@ -12185,6 +12185,72 @@
         </is>
       </c>
     </row>
+    <row r="114">
+      <c r="A114" s="16" t="n">
+        <v>46313.375</v>
+      </c>
+      <c r="B114" t="inlineStr">
+        <is>
+          <t>F09</t>
+        </is>
+      </c>
+      <c r="C114" t="inlineStr">
+        <is>
+          <t>Capability</t>
+        </is>
+      </c>
+      <c r="D114" t="inlineStr">
+        <is>
+          <t>[2026-10-18] Tonight / Tomorrow / Weekend / Next week + Select-the-date month calendar</t>
+        </is>
+      </c>
+      <c r="E114" t="inlineStr">
+        <is>
+          <t>Partial</t>
+        </is>
+      </c>
+      <c r="F114" t="inlineStr">
+        <is>
+          <t>Critical</t>
+        </is>
+      </c>
+      <c r="G114" t="inlineStr">
+        <is>
+          <t>Moderate</t>
+        </is>
+      </c>
+      <c r="H114" t="inlineStr">
+        <is>
+          <t>Remaining: compute Tonight/Tomorrow/Weekend/Next week ranges in the destination timezone (calendar day counts already group by venue-local day).</t>
+        </is>
+      </c>
+      <c r="I114" t="inlineStr">
+        <is>
+          <t>2026-10-18: Scrolling 14-day strip removed. New 'Select the date' chip in the When row opens a month calendar (big black date, small dark-green event count; month + year nav; past months blocked). Counts come from new GET /api/v1/explore/events/calendar (SQL GROUP BY venue-local day over the visibility CTE, no page cap; unsupported city -&gt; supported:false and client counts its loaded pool). Picking a day refetches the hub for exactly that day; cards drop the 'Tonight' label while a day is active. Verified /explore (Hermosa, Chicago): Oct 23 = 54 (strip showed 1), Nov 14 pick -&gt; 3 events + places. pytest 991 passed/36 skipped; Explore Vitest 156/30; full Vitest 557/122; tsc 0. Gap: When-chip ranges still use the browser clock, not destination timezone. 2026-09-25: Phase A calendar strip under When row on /explore; days with dated events only; day tap filters feed (events on day + places). Category chips hide at zero. 14-day client fetch widen; no new API. Vitest 107/18. Full month/provider calendar still open.</t>
+        </is>
+      </c>
+      <c r="J114" t="inlineStr">
+        <is>
+          <t>See related gates</t>
+        </is>
+      </c>
+      <c r="K114" t="inlineStr">
+        <is>
+          <t>Feature</t>
+        </is>
+      </c>
+      <c r="L114" t="inlineStr">
+        <is>
+          <t>Owner request: remove scroll strip; month calendar with per-day counts, month/year nav.</t>
+        </is>
+      </c>
+      <c r="M114" t="inlineStr"/>
+      <c r="N114" t="inlineStr">
+        <is>
+          <t>Explorer</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>

</xml_diff>